<commit_message>
fix(cart): refine business rules from gift to attached add-on accessory with dynamic pricing
</commit_message>
<xml_diff>
--- a/thuyttdoc/Kich_Ban_Ky_Thuat_Play4_Charm.xlsx
+++ b/thuyttdoc/Kich_Ban_Ky_Thuat_Play4_Charm.xlsx
@@ -528,25 +528,25 @@
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BẢNG ĐẶC TẢ KỊCH BẢN GIỎ HÀNG - CHUẨN NGHIỆP VỤ &amp; KINH DOANH (TECH SPEC)</t>
+          <t>BẢNG ĐẶC TẢ KỊCH BẢN GIỎ HÀNG: MUA KÈM PHỤ KIỆN (ATTACHED ADD-ON)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dự án: FPT Camera Play 4 &amp; Phụ kiện Charm Promo Engine | Chuẩn hóa theo góc nhìn Senior BA &amp; Product Owner</t>
+          <t>Dự án: FPT Camera Play 4 &amp; Phụ kiện Charm Add-on Engine | Bản chất: Mua kèm có điều kiện với giá ưu đãi (cấu hình linh hoạt)</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>PHẦN 1: 1. TỔ HỢP SỐ LƯỢNG (BASIC 1:1)</t>
+          <t>PHẦN 1: 1. TỔ HỢP SỐ LƯỢNG MUA KÈM (TỶ LỆ 1:1 CHUẨN)</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -617,12 +617,12 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>1. Tổ hợp số lượng (Basic 1:1)</t>
+          <t>1. Tổ hợp số lượng mua kèm (Tỷ lệ 1:1 chuẩn)</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Mua đúng tỷ lệ 1:1: Mua 1 Camera Play 4 và chọn 1 Charm tiêu chuẩn (Basic)</t>
+          <t>Mua đúng tỷ lệ 1:1: Mua 1 Camera Play 4 và chọn mua kèm 1 Charm tiêu chuẩn (Basic)</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -632,17 +632,17 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Mua 1 Camera Play 4 kích hoạt quyền mua 1 Charm tiêu chuẩn với giá 0đ. Hạn mức Charm 0đ tối đa = Số lượng Camera trong giỏ hàng (1 Cam = 1 Charm 0đ).</t>
+          <t>1 Camera Play 4 kích hoạt 01 suất mua kèm 01 Charm tiêu chuẩn với mức giá mua kèm ưu đãi (hiện tại áp dụng 0đ, có thể cấu hình linh hoạt). Hạn mức mua kèm giá ưu đãi = Số lượng Camera trong giỏ hàng (1 Cam = 1 suất mua kèm ưu đãi).</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Nếu mẫu Charm tiêu chuẩn khách chọn bị hết hàng: Cho phép khách chọn sang mẫu Charm tiêu chuẩn khác còn hàng.</t>
+          <t>Nếu mẫu Charm tiêu chuẩn khách chọn bị hết hàng: Cho phép khách chọn đổi sang mẫu Charm tiêu chuẩn khác còn hàng trong hạn mức mua kèm.</t>
         </is>
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>Đội Kinh doanh có muốn giới hạn số lượng Camera tối đa được mua kèm Charm 0đ trên mỗi đơn hàng không (VD: Tối đa 5 Cam/đơn để tránh gom hàng)?</t>
+          <t>Đội Kinh doanh dự kiến trong tương lai mức giá mua kèm ưu đãi này sẽ giữ 0đ hay chuyển sang thu phí ưu đãi (ví dụ: mua kèm với giá 29k, 49k)?</t>
         </is>
       </c>
     </row>
@@ -657,32 +657,32 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>1. Tổ hợp số lượng (Basic 1:1)</t>
+          <t>1. Tổ hợp số lượng mua kèm (Tỷ lệ 1:1 chuẩn)</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Vượt hạn mức (Cùng mẫu): Mua 1 Cam, khách chọn 2 Charm cùng Mẫu A</t>
+          <t>Vượt hạn mức mua kèm (Cùng mẫu): Mua 1 Cam, khách chọn 2 Charm cùng Mẫu A</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Đã có 1 Camera và 1 Charm A (0đ) trong giỏ. Khách bấm chọn thêm 1 Charm A nữa.</t>
+          <t>Đã có 1 Camera và 1 Charm A (giá mua kèm ưu đãi 0đ) trong giỏ. Khách bấm chọn thêm 1 Charm A nữa.</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Tách 2 Charm A thành 2 dòng riêng: 01 chiếc tính giá 0đ (theo Camera), 01 chiếc tính giá bán lẻ gốc niêm yết 150.000đ. Không tính giá trung bình cộng.</t>
+          <t>Tách 2 Charm A thành 2 dòng riêng: 01 chiếc tính theo giá mua kèm ưu đãi (hiện tại 0đ, theo hạn mức Camera), 01 chiếc tính giá bán lẻ gốc niêm yết 150.000đ. Không tính giá trung bình cộng.</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>Nếu khách bấm giảm bớt 1 Charm A: Hệ thống luôn ưu tiên giữ lại chiếc 0đ cho khách, bỏ chiếc tính tiền.</t>
+          <t>Nếu khách bấm giảm bớt 1 Charm A: Hệ thống luôn ưu tiên giữ lại chiếc hưởng giá mua kèm ưu đãi cho khách, bỏ chiếc tính giá bán lẻ.</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Khi khách chọn vượt quá số lượng 0đ, Kinh doanh muốn hệ thống tự động tính giá bán lẻ món thứ 2 hay hiển thị thông báo chặn không cho chọn thêm?</t>
+          <t>Khi khách chọn vượt quá số lượng mua kèm ưu đãi, Kinh doanh muốn hệ thống tự động tính giá bán lẻ chiếc thứ 2 hay hiển thị cảnh báo giới hạn?</t>
         </is>
       </c>
     </row>
@@ -697,32 +697,32 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>1. Tổ hợp số lượng (Basic 1:1)</t>
+          <t>1. Tổ hợp số lượng mua kèm (Tỷ lệ 1:1 chuẩn)</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Vượt hạn mức (Khác mẫu - Khác giá): Mua 1 Cam, chọn 1 Charm A (100k) và 1 Charm B (150k)</t>
+          <t>Vượt hạn mức mua kèm (Khác mẫu - Khác giá): Mua 1 Cam, chọn 1 Charm A (100k) và 1 Charm B (150k)</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>1 Camera Play 4 trong giỏ, khách tick chọn 1 Charm A (giá gốc 100k) và 1 Charm B (giá gốc 150k).</t>
+          <t>1 Camera Play 4 trong giỏ, khách tick chọn 1 Charm A (giá bán lẻ 100k) và 1 Charm B (giá bán lẻ 150k).</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Ưu tiên quyền lợi tốt nhất cho khách (Best-deal): Tự động tặng 0đ cho Charm có giá trị cao nhất (Charm B - 150k), Charm còn lại (Charm A - 100k) tính giá bán lẻ gốc.</t>
+          <t>Ưu tiên quyền lợi tốt nhất cho khách (Best-deal): Tự động áp dụng giá mua kèm ưu đãi (0đ) cho Charm có giá trị cao nhất (Charm B - 150k), Charm còn lại (Charm A - 100k) tính theo giá bán lẻ gốc.</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>Nếu khách bỏ chọn Charm B: Hệ thống tự động chuyển Charm A thành 0đ ngay lập tức để bảo vệ quyền lợi quà tặng của khách.</t>
+          <t>Nếu khách bỏ chọn Charm B: Hệ thống tự động chuyển Charm A sang hưởng suất mua kèm ưu đãi ngay lập tức.</t>
         </is>
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>Kinh doanh muốn ưu tiên tặng món có giá trị cao nhất (Best-deal for Customer) để tăng độ hài lòng, hay tặng món rẻ nhất để tối ưu chi phí quà tặng cho công ty?</t>
+          <t>Kinh doanh muốn ưu tiên áp dụng giá mua kèm ưu đãi cho món có giá trị cao nhất (Best-deal) hay món có giá trị thấp nhất để tối ưu doanh thu phụ kiện?</t>
         </is>
       </c>
     </row>
@@ -737,32 +737,32 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>1. Tổ hợp số lượng (Basic 1:1)</t>
+          <t>1. Tổ hợp số lượng mua kèm (Tỷ lệ 1:1 chuẩn)</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Dưới hạn mức: Mua 3 Camera nhưng khách chỉ chọn 1 Charm Mẫu A</t>
+          <t>Dưới hạn mức mua kèm: Mua 3 Camera nhưng khách chỉ chọn mua kèm 1 Charm Mẫu A</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Giỏ hàng có 3 Camera (được 3 suất Charm 0đ), nhưng khách chỉ chọn 1 Charm A.</t>
+          <t>Giỏ hàng có 3 Camera (được 3 suất mua kèm ưu đãi), nhưng khách chỉ chọn mua kèm 1 Charm A.</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>Không ép buộc mua đủ số lượng quà. Khách có toàn quyền mua ít hơn hạn mức. Hệ thống hiển thị lời nhắc nhẹ nhàng nhưng không chặn luồng thanh toán.</t>
+          <t>Không ép buộc mua đủ số lượng mua kèm. Khách có toàn quyền mua ít hơn hạn mức. Hệ thống hiển thị lời nhắc gợi ý mua kèm nhưng không chặn luồng thanh toán.</t>
         </is>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Khách bỏ qua lời nhắc và thanh toán: Đơn hàng chỉ xuất 3 Camera + 1 Charm. Quyền nhận 2 Charm còn lại sẽ hết hiệu lực khi đơn hoàn tất.</t>
+          <t>Khách bỏ qua lời nhắc và thanh toán: Đơn hàng chỉ xuất 3 Camera + 1 Charm. Quyền mua kèm ưu đãi của 2 Charm còn lại sẽ hết hiệu lực khi đơn hàng hoàn tất.</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Có cần gửi email/SMS nhắc nhở tặng voucher bù cho 2 suất quà khách chưa chọn không, hay mặc định khách tự nguyện từ bỏ quà tặng?</t>
+          <t>Có cần gửi thông báo nhắc khách vẫn còn suất mua phụ kiện giá ưu đãi không, hay để khách tự quyết định không mua kèm?</t>
         </is>
       </c>
     </row>
@@ -777,32 +777,32 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>1. Tổ hợp số lượng (Basic 1:1)</t>
+          <t>1. Tổ hợp số lượng mua kèm (Tỷ lệ 1:1 chuẩn)</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Không chọn quà: Mua 2 Camera nhưng không chọn bất kỳ Charm nào</t>
+          <t>Không mua kèm phụ kiện: Mua 2 Camera nhưng không chọn bất kỳ Charm nào</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Có 2 Camera Play 4 trong giỏ, khách không chọn phụ kiện nào và bấm đi đến thanh toán.</t>
+          <t>Có 2 Camera Play 4 trong giỏ, khách không chọn phụ kiện mua kèm nào và bấm đi đến thanh toán.</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Ưu đãi Charm 0đ là chính sách 'Mua Kèm Ngay', KHÔNG quy đổi thành tiền mặt, KHÔNG tự động bảo lưu thành voucher cho đơn hàng sau.</t>
+          <t>Chính sách mua kèm là ưu đãi 'Mua Kèm Ngay Cùng Đơn' (Instant Add-on), KHÔNG quy đổi thành tiền mặt, KHÔNG tự động bảo lưu thành voucher mua phụ kiện ở đơn hàng sau.</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>Tại bước thanh toán: Hiển thị hộp thoại xác nhận ngắn: 'Bạn đang bỏ qua 2 Charm 0đ tặng kèm. Bạn có muốn chọn quà ngay không?'.</t>
+          <t>Tại bước thanh toán: Hiển thị bảng xác nhận nhanh: 'Bạn đang không chọn phụ kiện mua kèm giá ưu đãi. Bạn có muốn chọn thêm phụ kiện trước khi thanh toán?'.</t>
         </is>
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>Kinh doanh có đồng ý cho phép khách bỏ qua quà tặng không, và nếu sau này khách gọi lên tổng đài khiếu nại đòi quà thì CSKH xử lý thế nào?</t>
+          <t>Nếu sau này khách nhận Camera rồi mới muốn mua bổ sung phụ kiện theo giá mua kèm ưu đãi thì CSKH có hỗ trợ tạo đơn bổ sung không?</t>
         </is>
       </c>
     </row>
@@ -817,32 +817,32 @@
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>1. Tổ hợp số lượng (Basic 1:1)</t>
+          <t>1. Tổ hợp số lượng mua kèm (Tỷ lệ 1:1 chuẩn)</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Giảm số lượng Camera (Đồng bộ ngược): Đang có 2 Cam + 2 Charm A (0đ), giảm Cam xuống 1</t>
+          <t>Giảm số lượng Camera (Đồng bộ ngược): Đang có 2 Cam + 2 Charm A (giá ưu đãi), giảm Cam xuống 1</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Giỏ hàng có 2 Camera + 2 Charm A (cả 2 đều 0đ). Khách bấm giảm bớt 1 Camera.</t>
+          <t>Giỏ hàng có 2 Camera + 2 Charm A (cả 2 đều giá mua kèm ưu đãi 0đ). Khách bấm giảm bớt 1 Camera.</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Suất ưu đãi 0đ giảm từ 2 xuống 1. Giữ nguyên 2 Charm A trong giỏ nhưng chiếc thứ 2 tự động chuyển thành tính giá niêm yết (150.000đ). Không tự ý xóa hàng của khách.</t>
+          <t>Hạn mức mua kèm ưu đãi giảm từ 2 xuống 1. Giữ nguyên 2 Charm A trong giỏ nhưng chiếc thứ 2 tự động chuyển thành tính giá bán lẻ niêm yết (150.000đ). Không tự ý xóa sản phẩm của khách.</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>Khách có quyền bấm xóa dòng Charm tính tiền 150.000đ nếu không có nhu cầu mua thêm.</t>
+          <t>Khách có quyền bấm xóa dòng Charm tính giá bán lẻ 150.000đ nếu không có nhu cầu mua thêm ngoài hạn mức.</t>
         </is>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>Kinh doanh muốn giữ lại Charm và chuyển sang tính giá gốc, hay tự động xóa bớt 1 Charm để giỏ hàng chỉ còn đúng 1 Camera + 1 Charm 0đ?</t>
+          <t>Kinh doanh muốn giữ lại phụ kiện và chuyển sang giá bán lẻ, hay tự động giảm số lượng phụ kiện mua kèm tương ứng với số Camera?</t>
         </is>
       </c>
     </row>
@@ -857,32 +857,32 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>1. Tổ hợp số lượng (Basic 1:1)</t>
+          <t>1. Tổ hợp số lượng mua kèm (Tỷ lệ 1:1 chuẩn)</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Giảm Camera khi đang chọn nhiều mẫu khác nhau: Đang có 2 Cam + 1 Charm A + 1 Charm B, giảm Cam xuống 1</t>
+          <t>Giảm Camera khi đang chọn nhiều mẫu phụ kiện khác nhau: Đang có 2 Cam + 1 Charm A + 1 Charm B, giảm Cam xuống 1</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Giỏ có 2 Cam + 1 Charm A (0đ) + 1 Charm B (0đ). Khách giảm Camera xuống 1.</t>
+          <t>Giỏ có 2 Cam + 1 Charm A + 1 Charm B (cả 2 đều giá ưu đãi 0đ). Khách giảm Camera xuống 1.</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Chỉ còn 1 suất 0đ: Giữ món có giá trị cao nhất làm 0đ, món còn lại tính giá gốc. Nếu 2 món bằng giá, giữ món khách chọn trước làm 0đ.</t>
+          <t>Hạn mức ưu đãi chỉ còn 1: Giữ món có giá bán lẻ cao nhất hưởng giá mua kèm ưu đãi (0đ), món còn lại chuyển về giá bán lẻ gốc. Nếu 2 món bằng giá, ưu tiên món khách đã chọn trước.</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Cho phép khách nhấp chuột trực tiếp vào lựa chọn để hoán đổi quyền 0đ giữa Mẫu A và Mẫu B một cách dễ dàng.</t>
+          <t>Cho phép khách nhấp chuột trực tiếp để hoán đổi quyền hưởng giá ưu đãi giữa Mẫu A và Mẫu B một cách dễ dàng.</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>Khi giảm số lượng Camera, Kinh doanh muốn hệ thống tự động chọn món 0đ theo quy tắc có sẵn hay bắt buộc bật bảng hỏi để khách tự tay chọn?</t>
+          <t>Khi giảm số lượng Camera, Kinh doanh muốn hệ thống tự động gán ưu đãi theo thuật toán hay bật bảng hỏi để khách tự chọn mẫu được hưởng ưu đãi?</t>
         </is>
       </c>
     </row>
@@ -897,32 +897,32 @@
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>1. Tổ hợp số lượng (Basic 1:1)</t>
+          <t>1. Tổ hợp số lượng mua kèm (Tỷ lệ 1:1 chuẩn)</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Mua số lượng lớn: Khách mua 10 Camera, muốn chia quà cho cả 3 mẫu Charm A, B, C</t>
+          <t>Mua số lượng lớn: Khách mua 10 Camera, muốn chia phụ kiện mua kèm cho cả 3 mẫu Charm A, B, C</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Khách mua số lượng lớn (10 Camera Play 4, được 10 suất Charm 0đ).</t>
+          <t>Khách mua số lượng lớn (10 Camera Play 4, được 10 suất mua kèm phụ kiện giá ưu đãi).</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>Cho phép khách gõ trực tiếp số lượng từng mẫu Charm vào ô nhập liệu (thay vì bấm nút [+] 10 lần). Tổng số lượng Charm 0đ không vượt quá 10.</t>
+          <t>Cho phép khách nhập trực tiếp số lượng từng mẫu phụ kiện mua kèm vào ô số lượng. Tổng số lượng Charm hưởng giá mua kèm ưu đãi tối đa không vượt quá 10 chiếc.</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>Hiển thị thanh tiến trình trực quan: 'Đã phân bổ: 7/10 Charm 0đ'. Nếu nhập quá 10, số lượng vượt sẽ tự động tính theo giá bán lẻ.</t>
+          <t>Hiển thị thanh tiến trình trực quan: 'Đã phân bổ: 7/10 phụ kiện mua kèm ưu đãi'. Nếu nhập vượt quá 10, số lượng dư ra sẽ tự động tính theo giá bán lẻ.</t>
         </is>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>Chính sách mua số lượng lớn (trên 10 chiếc) áp dụng cho khách hàng cá nhân hay có kênh bán hàng sỉ/B2B riêng với mức chiết khấu khác?</t>
+          <t>Chính sách mua kèm số lượng lớn (trên 10 thiết bị) có áp dụng chung chính sách mua kèm này hay áp dụng theo báo giá đại lý/B2B riêng?</t>
         </is>
       </c>
     </row>
@@ -937,22 +937,22 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>1. Tổ hợp số lượng (Basic 1:1)</t>
+          <t>1. Tổ hợp số lượng mua kèm (Tỷ lệ 1:1 chuẩn)</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Đổi mẫu phụ kiện: Đang có 3 Cam + 3 Charm (1A, 1B, 1C), muốn đổi C thành A</t>
+          <t>Đổi mẫu phụ kiện mua kèm: Đang chọn 3 Cam + 3 Charm (1A, 1B, 1C), muốn đổi C thành A</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Đã chọn tối đa 3 Charm (1A, 1B, 1C). Suất quà 0đ khả dụng = 0.</t>
+          <t>Đã chọn tối đa 3 Charm mua kèm (1A, 1B, 1C). Hạn mức mua kèm ưu đãi khả dụng = 0.</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>Khi khách giảm số lượng Mẫu C về 0, suất 0đ ngay lập tức được giải phóng. Khách bấm tăng Mẫu A lên 2 chiếc thì chiếc thứ 2 được hưởng giá 0đ.</t>
+          <t>Khi khách giảm số lượng Mẫu C về 0, hạn mức mua kèm ưu đãi lập tức được giải phóng. Khách bấm tăng Mẫu A lên 2 chiếc thì chiếc thứ 2 được áp dụng giá mua kèm ưu đãi.</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="H14" s="9" t="inlineStr">
         <is>
-          <t>Trải nghiệm đổi quà nên diễn ra trực tiếp tại giỏ hàng hay cần nút 'Đổi quà tặng' chuyên biệt để khách thao tác thuận tiện nhất?</t>
+          <t>Giao diện đổi mẫu phụ kiện mua kèm có cần hiển thị nút 'Đổi mẫu mua kèm' trực tiếp tại từng dòng sản phẩm không?</t>
         </is>
       </c>
     </row>
@@ -977,39 +977,39 @@
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>1. Tổ hợp số lượng (Basic 1:1)</t>
+          <t>1. Tổ hợp số lượng mua kèm (Tỷ lệ 1:1 chuẩn)</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Xóa Camera khỏi giỏ: Đang có 1 Cam + 1 Charm 0đ, khách bấm xóa Camera</t>
+          <t>Xóa Camera khỏi giỏ: Đang có 1 Cam + 1 Charm mua kèm, khách bấm xóa Camera</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Có 1 Camera Play 4 + 1 Charm 0đ trong giỏ hàng. Khách bấm nút 'Xóa' Camera.</t>
+          <t>Có 1 Camera Play 4 + 1 Charm mua kèm giá ưu đãi trong giỏ. Khách bấm nút 'Xóa' Camera.</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>Quy tắc ràng buộc: Charm 0đ không thể tồn tại độc lập khi không có Camera. Xóa Camera sẽ làm mất điều kiện nhận quà tặng 0đ.</t>
+          <t>Quy tắc ràng buộc chặt (Strict Binding): Phụ kiện mua kèm giá ưu đãi không thể tồn tại độc lập khi không có sản phẩm chính. Xóa Camera đồng nghĩa mất điều kiện mua kèm giá ưu đãi.</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>Hệ thống hỏi khách: 'Xóa Camera sẽ mất quà tặng 0đ. Bạn có muốn giữ lại Charm với giá bán lẻ 150.000đ không? [Xóa tất cả] [Giữ Charm giá gốc]'.</t>
+          <t>Hệ thống hỏi khách: 'Xóa Camera sẽ mất quyền mua phụ kiện giá ưu đãi. Bạn có muốn giữ lại phụ kiện với giá bán lẻ 150.000đ không? [Xóa tất cả] [Giữ Charm giá bán lẻ]'.</t>
         </is>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>Kinh doanh muốn tự động xóa sạch Charm đi kèm khi xóa Camera, hay giữ lại Charm và thông báo tính giá gốc?</t>
+          <t>Kinh doanh muốn tự động xóa toàn bộ phụ kiện mua kèm khi xóa Camera chính, hay giữ lại phụ kiện và chuyển sang giá bán lẻ?</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>PHẦN 2: 2. PHỤ THU NÂNG CẤP (CHARM PREMIUM +50K)</t>
+          <t>PHẦN 2: 2. PHỤ THU NÂNG CẤP PHỤ KIỆN (CHARM PREMIUM +50K)</t>
         </is>
       </c>
       <c r="B16" s="5" t="n"/>
@@ -1031,32 +1031,32 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>2. Phụ thu nâng cấp (Charm Premium +50k)</t>
+          <t>2. Phụ thu nâng cấp phụ kiện (Charm Premium +50k)</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Mua kết hợp Bản thường &amp; Bản cao cấp: Mua 2 Cam, chọn 1 Charm Basic (0đ) + 1 Charm Premium (+50k)</t>
+          <t>Mua kèm kết hợp Bản tiêu chuẩn &amp; Bản nâng cấp: Mua 2 Cam, chọn 1 Charm Basic + 1 Charm Premium</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>2 Camera Play 4 (được 2 suất ưu đãi). Kho còn cả mẫu Basic và mẫu Premium.</t>
+          <t>2 Camera Play 4 (được 2 suất mua kèm ưu đãi). Kho còn cả mẫu Basic và mẫu Premium.</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>1 Camera được đổi 1 Charm tiêu chuẩn 0đ HOẶC nâng cấp lên Charm Premium với mức phụ thu ưu đãi +50.000đ/chiếc (thay vì giá bán lẻ gốc 200.000đ).</t>
+          <t>Mỗi Camera cho phép mua kèm 1 Charm tiêu chuẩn với giá ưu đãi (hiện tại 0đ) HOẶC nâng cấp lên Charm Premium với mức giá phụ thu ưu đãi +50.000đ/chiếc (thay vì giá bán lẻ gốc 200.000đ). Mức phụ thu này có thể cấu hình linh hoạt.</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>Hóa đơn hiển thị rõ: Tiền Camera + Phụ thu nâng cấp Charm Premium 50.000đ (Tiết kiệm 150.000đ).</t>
+          <t>Bảng kê đơn hàng hiển thị rõ: Tiền Camera + Phụ thu nâng cấp Charm Premium 50.000đ (Tiết kiệm 150.000đ so với giá bán lẻ).</t>
         </is>
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>Khoản thu 50.000đ này kế toán sẽ ghi nhận vào doanh thu phụ kiện Charm hay phân bổ giảm trừ vào giá bán của Camera?</t>
+          <t>Khoản thu 50.000đ này kế toán sẽ ghi nhận vào doanh thu bán lẻ phụ kiện hay phân bổ tính vào gói sản phẩm Camera?</t>
         </is>
       </c>
     </row>
@@ -1071,32 +1071,32 @@
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>2. Phụ thu nâng cấp (Charm Premium +50k)</t>
+          <t>2. Phụ thu nâng cấp phụ kiện (Charm Premium +50k)</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>Vượt hạn mức kết hợp: Mua 1 Cam, chọn cả 1 Charm Basic + 1 Charm Premium</t>
+          <t>Vượt hạn mức khi chọn cả 2 loại: Mua 1 Cam, chọn cả 1 Charm Basic + 1 Charm Premium</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>1 Camera Play 4 (chỉ có 1 suất ưu đãi). Khách chọn 2 món phụ kiện khác loại.</t>
+          <t>1 Camera Play 4 (chỉ có 1 suất mua kèm ưu đãi). Khách chọn 2 phụ kiện khác phân khúc.</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Áp dụng suất ưu đãi cho món mang lại quyền lợi cao nhất: Charm Basic 0đ + Charm Premium tính giá bán lẻ gốc 200k (Tổng tiền phụ kiện = 200k).</t>
+          <t>Áp dụng suất mua kèm ưu đãi cho món mang lại quyền lợi cao nhất: Charm Basic giá ưu đãi 0đ + Charm Premium tính giá bán lẻ gốc 200k (Tổng tiền phụ kiện = 200k).</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>Nếu khách muốn áp dụng suất ưu đãi cho Premium (trả 50k) và trả tiền gốc cho Basic (150k): Tổng tiền phụ kiện vẫn là 200k.</t>
+          <t>Nếu khách muốn áp dụng suất ưu đãi cho Premium (phụ thu 50k) và trả tiền gốc cho Basic (150k): Tổng tiền phụ kiện vẫn là 200k.</t>
         </is>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>Kinh doanh có đồng ý cho khách chủ động chọn món nào được hưởng ưu đãi (Basic 0đ hay Premium 50k) trong trường hợp này không?</t>
+          <t>Kinh doanh có đồng ý cho khách chủ động chọn món nào được hưởng suất mua kèm ưu đãi (Basic hay Premium) trong trường hợp này không?</t>
         </is>
       </c>
     </row>
@@ -1111,32 +1111,32 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>2. Phụ thu nâng cấp (Charm Premium +50k)</t>
+          <t>2. Phụ thu nâng cấp phụ kiện (Charm Premium +50k)</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Đổi ý nâng cấp (Swap): Đang chọn Charm Basic 0đ, khách bấm đổi sang Charm Premium</t>
+          <t>Đổi ý nâng cấp (Swap): Đang chọn Charm Basic, khách bấm đổi sang Charm Premium</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Giỏ có 1 Cam + 1 Charm Basic 0đ. Khách tick chọn sang mẫu Premium.</t>
+          <t>Giỏ có 1 Cam + 1 Charm Basic giá ưu đãi 0đ. Khách tick chọn sang mẫu Premium.</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>Hệ thống tự động hủy chọn mẫu Basic và áp dụng mức phụ thu +50.000đ cho mẫu Premium. Tổng số tiền thanh toán tăng thêm đúng 50.000đ.</t>
+          <t>Hệ thống tự động hủy chọn mẫu Basic và kích hoạt mức giá mua kèm ưu đãi cho Premium (phụ thu +50.000đ). Tổng tiền thanh toán tăng thêm đúng 50.000đ.</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Giao diện cập nhật tức thì, có thông báo: 'Đã nâng cấp lên phiên bản Charm Premium (+50.000đ)'.</t>
+          <t>Giao diện cập nhật tức thì kèm thông báo: 'Đã chuyển sang mua kèm phiên bản phụ kiện Premium (+50.000đ)'.</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>Có cần làm nổi bật lợi ích 'Chỉ thêm 50k sở hữu ngay bản Giới hạn/Cao cấp' để kích thích khách hàng nâng cấp (Upsell) không?</t>
+          <t>Có cần thiết kế nhãn 'Nâng cấp chỉ +50k' nổi bật để thúc đẩy doanh thu bán kèm phụ kiện cao cấp (Upsell) không?</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>2. Phụ thu nâng cấp (Charm Premium +50k)</t>
+          <t>2. Phụ thu nâng cấp phụ kiện (Charm Premium +50k)</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
@@ -1166,17 +1166,17 @@
       </c>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>Giữ nguyên 1 Charm Premium (+50k) và mở thêm 01 ô quà tặng còn trống để khách tự do chọn thêm món thứ 2. KHÔNG tự động nhân đôi Premium thành 2 cái (+100k).</t>
+          <t>Giữ nguyên 1 Charm Premium (+50k) và mở thêm 01 suất mua kèm ưu đãi còn trống để khách tự do chọn thêm món thứ 2. KHÔNG tự ý nhân đôi Premium thành 2 cái (+100k).</t>
         </is>
       </c>
       <c r="G20" s="12" t="inlineStr">
         <is>
-          <t>Khách có thể chọn thêm 1 Charm Basic (0đ) hoặc thêm 1 Charm Premium (+50k) tùy nhu cầu.</t>
+          <t>Khách có thể chọn thêm 1 Charm Basic (giá ưu đãi 0đ) hoặc thêm 1 Charm Premium (+50k) theo nhu cầu.</t>
         </is>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>Khi khách tăng Camera, Kinh doanh muốn hệ thống gợi ý chọn thêm quà ngay hay để khách tự vào giỏ hàng chọn sau?</t>
+          <t>Khi khách tăng số lượng Camera, Kinh doanh muốn hệ thống gợi ý chọn thêm phụ kiện mua kèm ngay hay để khách tự chọn trong giỏ hàng?</t>
         </is>
       </c>
     </row>
@@ -1191,32 +1191,32 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>2. Phụ thu nâng cấp (Charm Premium +50k)</t>
+          <t>2. Phụ thu nâng cấp phụ kiện (Charm Premium +50k)</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Giảm Camera khi đang có cả 2 loại: Đang có 2 Cam + 1 Basic (0đ) + 1 Premium (+50k), giảm Cam xuống 1</t>
+          <t>Giảm Camera khi đang có cả 2 loại: Đang có 2 Cam + 1 Basic + 1 Premium (+50k), giảm Cam xuống 1</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Giỏ có 2 Cam + 1 Basic + 1 Premium. Khách bấm [-] giảm Camera về 1.</t>
+          <t>Giỏ có 2 Cam + 1 Basic (0đ) + 1 Premium (+50k). Khách bấm [-] giảm Camera về 1.</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Suất ưu đãi giảm còn 1: Ưu tiên giữ lại suất Charm Basic 0đ, chiếc Charm Premium chuyển sang tính theo giá bán lẻ gốc 200.000đ.</t>
+          <t>Hạn mức ưu đãi giảm còn 1: Ưu tiên giữ lại suất ưu đãi cho Charm Basic (0đ), chiếc Charm Premium chuyển sang tính theo giá bán lẻ gốc 200.000đ.</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>Hiển thị thông báo nhanh cho khách chọn: 'Giữ Charm Basic 0đ' hoặc 'Giữ Charm Premium ưu đãi 50k (bỏ Basic)'.</t>
+          <t>Hiển thị thông báo nhanh cho khách chọn: 'Áp dụng ưu đãi cho Charm Basic (0đ)' hoặc 'Áp dụng ưu đãi cho Charm Premium (50k)'.</t>
         </is>
       </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>Kinh doanh muốn ưu tiên giữ suất miễn phí (0đ) hay giữ suất có phụ thu (+50k) khi khách giảm số lượng mua?</t>
+          <t>Kinh doanh muốn ưu tiên giữ suất mua kèm giá 0đ hay giữ suất có phụ thu (+50k) khi khách giảm số lượng mua thiết bị chính?</t>
         </is>
       </c>
     </row>
@@ -1231,39 +1231,39 @@
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>2. Phụ thu nâng cấp (Charm Premium +50k)</t>
+          <t>2. Phụ thu nâng cấp phụ kiện (Charm Premium +50k)</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>Chính sách đổi trả khi có phụ thu nâng cấp</t>
+          <t>Chính sách đổi trả Camera khi có mua kèm phụ kiện phụ thu nâng cấp</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Đơn hàng hoàn tất gồm 1 Camera Play 4 (800k) + 1 Charm Premium (50k). Khách muốn trả Camera, giữ lại Charm.</t>
+          <t>Đơn hàng hoàn tất gồm 1 Camera Play 4 (800k) + 1 Charm Premium mua kèm (50k). Khách muốn trả Camera, giữ lại Charm.</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
         <is>
-          <t>Khách trả Camera nhưng giữ Charm Premium: Charm không còn điều kiện mua kèm, bị tính theo giá bán lẻ gốc (200k). Số tiền hoàn lại = Tiền Camera (800k) - Chênh lệch Charm (200k - 50k = 150k) = 650.000đ.</t>
+          <t>Khách trả Camera nhưng giữ Charm Premium: Charm không còn điều kiện mua kèm ưu đãi, phải tính theo giá bán lẻ gốc (200k). Số tiền hoàn lại = Tiền Camera (800k) - Chênh lệch giá Charm (200k - 50k = 150k) = 650.000đ.</t>
         </is>
       </c>
       <c r="G22" s="12" t="inlineStr">
         <is>
-          <t>Nếu khách trả lại cả Camera và Charm Premium còn nguyên vẹn: Hoàn đủ 100% số tiền thực thu (850.000đ).</t>
+          <t>Nếu khách hoàn trả cả Camera và Charm Premium còn nguyên vẹn: Hoàn đủ 100% số tiền thực thu (850.000đ).</t>
         </is>
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>Kinh doanh có đồng ý với phương án cấn trừ tiền hoàn chênh lệch này không, hay bắt buộc khách phải trả đủ cả bộ mới được hoàn tiền?</t>
+          <t>Kinh doanh có đồng ý với nguyên tắc cấn trừ tiền hoàn này khi khách tách lẻ phụ kiện mua kèm không, hay bắt buộc phải trả trọn bộ mới giải quyết?</t>
         </is>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>PHẦN 3: 3. BÁN CHÉO SỐ LƯỢNG (MUA THÊM CHARM 2, 3 GIẢM 50%)</t>
+          <t>PHẦN 3: 3. BÁN CHÉO SỐ LƯỢNG (MUA THÊM PHỤ KIỆN THỨ 2, 3 GIẢM 50%)</t>
         </is>
       </c>
       <c r="B23" s="5" t="n"/>
@@ -1285,32 +1285,32 @@
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>3. Bán chéo số lượng (Mua thêm Charm 2, 3 giảm 50%)</t>
+          <t>3. Bán chéo số lượng (Mua thêm phụ kiện thứ 2, 3 giảm 50%)</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>Mua nhiều Charm giá khác nhau: 1 Cam, chọn 3 Charm giá gốc khác nhau (100k, 150k, 200k)</t>
+          <t>Mua kèm nhiều phụ kiện giá khác nhau: 1 Cam, chọn 3 Charm giá bán lẻ khác nhau (100k, 150k, 200k)</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Chính sách: Mua 1 Cam được 1 Charm 0đ + tối đa 2 Charm tiếp theo giảm 50%. Khách chọn 3 Charm (100k, 150k, 200k).</t>
+          <t>Chính sách: Mua 1 Cam được 1 Charm giá ưu đãi (hiện tại 0đ) + tối đa 2 Charm tiếp theo giảm 50%. Khách chọn 3 Charm (100k, 150k, 200k).</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>Ưu tiên tối đa quyền lợi khách hàng: Chiếc 200k tặng 0đ (tiết kiệm 200k). Chiếc 150k giảm 50% còn 75k. Chiếc 100k giảm 50% còn 50k. Tổng phụ kiện = 125k (Tiết kiệm 325k).</t>
+          <t>Ưu tiên quyền lợi lớn nhất cho khách: Chiếc 200k áp dụng giá mua kèm ưu đãi 0đ (tiết kiệm 200k). Chiếc 150k giảm 50% còn 75k. Chiếc 100k giảm 50% còn 50k. Tổng tiền phụ kiện = 125k (Tiết kiệm 325k).</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Nếu chính sách kinh doanh ưu tiên bảo vệ lợi nhuận: Tặng 0đ cho chiếc rẻ nhất (100k) và giảm 50% cho 2 chiếc còn lại.</t>
+          <t>Nếu chính sách kinh doanh ưu tiên bảo vệ biên lợi nhuận: Áp dụng giá ưu đãi 0đ cho chiếc rẻ nhất (100k) và giảm 50% cho 2 chiếc còn lại.</t>
         </is>
       </c>
       <c r="H24" s="9" t="inlineStr">
         <is>
-          <t>Kinh doanh lựa chọn phương án nào: Tối ưu lợi ích cho khách (giảm giá chiếc đắt nhất) hay Bảo vệ doanh thu (giảm giá chiếc rẻ nhất)?</t>
+          <t>Kinh doanh chọn phương án nào: Ưu đãi tốt nhất cho khách (giảm giá món đắt nhất) hay Bảo vệ doanh thu (giảm giá món rẻ nhất)?</t>
         </is>
       </c>
     </row>
@@ -1325,32 +1325,32 @@
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>3. Bán chéo số lượng (Mua thêm Charm 2, 3 giảm 50%)</t>
+          <t>3. Bán chéo số lượng (Mua thêm phụ kiện thứ 2, 3 giảm 50%)</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Vượt trần ưu đãi: Mua 1 Cam nhưng khách chọn tới 5 Charm</t>
+          <t>Vượt trần số lượng mua kèm ưu đãi: Mua 1 Cam nhưng khách chọn tới 5 Charm</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>1 Camera Play 4. Hạn mức tối đa: 1 Charm 0đ + 2 Charm giảm 50% (Tổng tối đa 3 chiếc có ưu đãi). Khách chọn 5 Charm.</t>
+          <t>1 Camera Play 4. Hạn mức tối đa: 1 Charm giá ưu đãi 0đ + 2 Charm giảm 50% (Tổng tối đa 3 chiếc hưởng giá mua kèm ưu đãi). Khách chọn 5 Charm.</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>Chiếc thứ 1: Tặng 0đ. Chiếc thứ 2 và 3: Giảm 50%. Chiếc thứ 4 và thứ 5: Tính nguyên giá bán lẻ 100%.</t>
+          <t>Chiếc thứ 1: Giá ưu đãi 0đ. Chiếc thứ 2 và 3: Giảm 50%. Chiếc thứ 4 và thứ 5: Tính nguyên giá bán lẻ niêm yết 100%.</t>
         </is>
       </c>
       <c r="G25" s="12" t="inlineStr">
         <is>
-          <t>Nếu khách mua thêm Camera thứ 2: Hạn mức mở rộng thành 2 chiếc 0đ + 4 chiếc 50%, chiếc thứ 4 và 5 tự động chuyển sang hưởng giảm 50% ngay.</t>
+          <t>Nếu khách mua thêm Camera thứ 2: Hạn mức mở rộng thành 2 chiếc 0đ + 4 chiếc 50%, chiếc thứ 4 và 5 tự động chuyển sang hưởng giảm 50% ngay lập tức.</t>
         </is>
       </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
-          <t>Giới hạn mua thêm giảm 50% nên chốt là tối đa 2 chiếc hay mở rộng theo tỷ lệ số Camera mua?</t>
+          <t>Chính sách giảm giá 50% cho phụ kiện thứ 2, thứ 3 có áp dụng xuyên suốt hay chỉ áp dụng trong các đợt chiến dịch khuyến mại nhất định?</t>
         </is>
       </c>
     </row>
@@ -1365,32 +1365,32 @@
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>3. Bán chéo số lượng (Mua thêm Charm 2, 3 giảm 50%)</t>
+          <t>3. Bán chéo số lượng (Mua thêm phụ kiện thứ 2, 3 giảm 50%)</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Xóa Camera khi đang có Charm 0đ và Charm giảm 50%</t>
+          <t>Xóa Camera khi đang có phụ kiện mua kèm giá ưu đãi và giảm 50%</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>Giỏ có 1 Camera + 1 Charm 0đ + 1 Charm giảm 50%. Khách xóa Camera khỏi giỏ.</t>
+          <t>Giỏ có 1 Camera + 1 Charm giá ưu đãi 0đ + 1 Charm giảm 50%. Khách xóa Camera khỏi giỏ.</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>Toàn bộ ưu đãi mua kèm bị vô hiệu lực. Hệ thống cảnh báo và chuyển toàn bộ các Charm về giá niêm yết 100% nếu khách muốn giữ giỏ, hoặc xóa toàn bộ.</t>
+          <t>Toàn bộ điều kiện mua kèm bị vô hiệu lực. Hệ thống cảnh báo và chuyển toàn bộ các Charm về giá bán lẻ niêm yết 100% nếu khách muốn giữ giỏ, hoặc xóa toàn bộ phụ kiện.</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>Bảng hỏi: 'Xóa Camera sẽ làm mất toàn bộ ưu đãi phụ kiện 0đ và giảm 50%. Bạn có muốn tiếp tục? [Xóa tất cả] [Giữ Charm giá gốc]'.</t>
+          <t>Hộp thoại xác nhận: 'Xóa Camera sẽ làm mất toàn bộ giá mua kèm ưu đãi của phụ kiện. Bạn có muốn tiếp tục? [Xóa tất cả] [Giữ Charm giá bán lẻ gốc]'.</t>
         </is>
       </c>
       <c r="H26" s="9" t="inlineStr">
         <is>
-          <t>Kinh doanh có muốn áp dụng mức giảm giá khác (VD: Giảm 10% khách hàng mới) nếu khách quyết định giữ lại phụ kiện không?</t>
+          <t>Kinh doanh có muốn áp dụng mức chiết khấu thông thường (VD: Giảm 10% phụ kiện lẻ) nếu khách vẫn muốn giữ lại mua phụ kiện sau khi xóa Camera không?</t>
         </is>
       </c>
     </row>
@@ -1405,32 +1405,32 @@
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>3. Bán chéo số lượng (Mua thêm Charm 2, 3 giảm 50%)</t>
+          <t>3. Bán chéo số lượng (Mua thêm phụ kiện thứ 2, 3 giảm 50%)</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Dịch chuyển thứ tầng ưu đãi khi giảm Camera: Giảm Cam từ 2 xuống 1</t>
+          <t>Dịch chuyển thứ tầng giá ưu đãi khi giảm Camera: Giảm Cam từ 2 xuống 1</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Giỏ có 2 Cam + 2 Charm (0đ) + 2 Charm (50%). Khách bấm giảm Camera xuống 1.</t>
+          <t>Giỏ có 2 Cam + 2 Charm (ưu đãi 0đ) + 2 Charm (giảm 50%). Khách bấm giảm Camera xuống 1.</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>Hạn mức mới: 1 Charm 0đ + 2 Charm 50% + 1 Charm giá gốc 100%. Hệ thống tự động dịch chuyển món đắt nhất vào nhóm 0đ, tiếp theo vào nhóm 50% và món rẻ nhất về giá gốc.</t>
+          <t>Hạn mức mới: 1 Charm ưu đãi 0đ + 2 Charm giảm 50% + 1 Charm tính giá bán lẻ gốc 100%. Hệ thống tự động dịch chuyển món đắt nhất vào nhóm 0đ, tiếp theo vào nhóm 50% và món còn lại về giá gốc.</t>
         </is>
       </c>
       <c r="G27" s="12" t="inlineStr">
         <is>
-          <t>Giá đơn hàng cập nhật tức thì kèm thông báo lý do điều chỉnh số lượng ưu đãi.</t>
+          <t>Tổng tiền đơn hàng cập nhật tức thì kèm thông báo giải thích việc điều chỉnh hạn mức mua kèm.</t>
         </is>
       </c>
       <c r="H27" s="13" t="inlineStr">
         <is>
-          <t>Quy tắc trượt tầng giá tự động này có đáp ứng đúng mong muốn vận hành của đội ngũ Kinh doanh không?</t>
+          <t>Quy tắc trượt tầng giá mua kèm tự động này có đúng với mong đợi vận hành của đội ngũ Kinh doanh không?</t>
         </is>
       </c>
     </row>
@@ -1445,39 +1445,39 @@
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>3. Bán chéo số lượng (Mua thêm Charm 2, 3 giảm 50%)</t>
+          <t>3. Bán chéo số lượng (Mua thêm phụ kiện thứ 2, 3 giảm 50%)</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>Đóng gói &amp; Giao nhận khi đơn hàng có nhiều mức giá khác nhau</t>
+          <t>Đóng gói &amp; Giao nhận khi đơn hàng có nhiều mức giá mua kèm khác nhau</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>Đơn hàng hoàn tất gồm 1 Cam + 1 Charm 0đ + 2 Charm giảm 50%.</t>
+          <t>Đơn hàng hoàn tất gồm 1 Cam + 1 Charm giá ưu đãi 0đ + 2 Charm giảm 50%.</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>Tất cả các sản phẩm được đóng chung trong CÙNG MỘT KIỆN HÀNG nếu xuất cùng một kho, không tách rời theo mức giá khuyến mãi.</t>
+          <t>Tất cả các sản phẩm được đóng chung trong CÙNG MỘT KIỆN HÀNG nếu xuất cùng một kho, không phân biệt phụ kiện mua kèm theo các mức giá khác nhau.</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>Hóa đơn và phiếu giao hàng ghi rõ từng dòng sản phẩm với đơn giá thực tế đã giảm để giao cho khách.</t>
+          <t>Hóa đơn và phiếu giao hàng ghi rõ từng dòng sản phẩm với đơn giá mua kèm thực tế để đối soát khi giao nhận.</t>
         </is>
       </c>
       <c r="H28" s="9" t="inlineStr">
         <is>
-          <t>Kho vận có yêu cầu dán tem phân biệt giữa phụ kiện tặng 0đ và phụ kiện bán lẻ giảm giá 50% không?</t>
+          <t>Kho vận có cần phân biệt tem nhãn giữa phụ kiện mua kèm giá 0đ và phụ kiện mua thêm giảm giá 50% không?</t>
         </is>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>PHẦN 4: 4. COMBO BOOSTER (BUNDLE PLAY4 + DÒNG KHÁC)</t>
+          <t>PHẦN 4: 4. COMBO BOOSTER (MUA KÈM KHI MUA GÓI COMBO THIẾT BỊ)</t>
         </is>
       </c>
       <c r="B29" s="5" t="n"/>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>4. Combo Booster (Bundle Play4 + Dòng khác)</t>
+          <t>4. Combo Booster (Mua kèm khi mua gói Combo thiết bị)</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -1514,17 +1514,17 @@
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>Do trong Combo có thiết bị Play 4, khách vẫn được kích hoạt đúng 01 suất mua Charm 0đ như khi mua lẻ.</t>
+          <t>Do trong Combo có chứa thiết bị Camera Play 4, khách vẫn được hưởng đầy đủ 01 suất mua kèm phụ kiện Charm với giá ưu đãi (hiện tại 0đ) như khi mua lẻ Play 4.</t>
         </is>
       </c>
       <c r="G30" s="12" t="inlineStr">
         <is>
-          <t>Trang chi tiết của Combo hiển thị rõ: 'Tặng kèm 01 Charm Play 4 tự chọn trị giá 150.000đ'.</t>
+          <t>Trang chi tiết của Combo hiển thị rõ: 'Ưu đãi mua kèm 01 Charm Play 4 với giá đặc biệt 0đ'.</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr">
         <is>
-          <t>Nếu mã Combo này đã được giảm giá sốc hơn 20%, Kinh doanh có muốn loại trừ quà tặng Charm 0đ không?</t>
+          <t>Nếu mã Combo này đã được giảm giá sốc hơn 20%, Kinh doanh có muốn loại trừ chính sách mua kèm phụ kiện giá ưu đãi không?</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>4. Combo Booster (Bundle Play4 + Dòng khác)</t>
+          <t>4. Combo Booster (Mua kèm khi mua gói Combo thiết bị)</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
@@ -1554,17 +1554,17 @@
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>Hệ thống tự động nhận diện cặp sản phẩm hợp lệ, áp dụng giá ưu đãi Combo (tiết kiệm thêm) và vẫn mở đầy đủ quyền nhận 01 Charm 0đ.</t>
+          <t>Hệ thống tự động nhận diện cặp sản phẩm hợp lệ để áp dụng giá ưu đãi Combo (nếu có), đồng thời vẫn bảo đảm 01 suất mua kèm Charm với giá ưu đãi.</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>Hiển thị thông báo: 'Đã tự động ghép Combo An Ninh - Tiết kiệm thêm 100k + Tặng 1 Charm 0đ'.</t>
+          <t>Hiển thị thông báo: 'Đã tự động ghép Combo An Ninh - Tiết kiệm thêm 100k + Ưu đãi mua kèm 1 Charm giá 0đ'.</t>
         </is>
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>Kinh doanh muốn hệ thống tự động ghép Combo để kích cầu hay bắt buộc khách phải chọn mua đúng link Combo mới được giảm giá?</t>
+          <t>Kinh doanh muốn hệ thống tự động ghép Combo kích cầu hay bắt buộc khách phải chọn mua đúng mã Combo được tạo sẵn?</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>4. Combo Booster (Bundle Play4 + Dòng khác)</t>
+          <t>4. Combo Booster (Mua kèm khi mua gói Combo thiết bị)</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
@@ -1589,22 +1589,22 @@
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Đang có Combo mềm trong giỏ và đã chọn Charm 0đ. Khách xóa chiếc IQ4S.</t>
+          <t>Đang có Combo mềm trong giỏ và đã chọn Charm mua kèm giá ưu đãi. Khách xóa chiếc IQ4S.</t>
         </is>
       </c>
       <c r="F32" s="12" t="inlineStr">
         <is>
-          <t>Combo bị hủy, Play 4 trở về giá bán lẻ thông thường. Quyền nhận 01 Charm 0đ theo Camera Play 4 vẫn ĐƯỢC GIỮ NGUYÊN.</t>
+          <t>Combo bị hủy, Play 4 quay về giá bán lẻ thông thường. Do Camera Play 4 vẫn có chính sách bán kèm phụ kiện nên suất mua kèm Charm giá ưu đãi VẪN ĐƯỢC GIỮ NGUYÊN.</t>
         </is>
       </c>
       <c r="G32" s="12" t="inlineStr">
         <is>
-          <t>Thông báo: 'Combo an ninh đã hủy do giảm sản phẩm. Giá Play 4 quay về giá gốc. Ưu đãi 1 Charm 0đ vẫn được giữ'.</t>
+          <t>Thông báo: 'Combo an ninh đã hủy do giảm bớt sản phẩm. Giá Play 4 quay về giá gốc. Suất mua kèm phụ kiện giá ưu đãi vẫn được bảo lưu'.</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr">
         <is>
-          <t>Nếu sau này có loại Combo mà chỉ khi mua Combo mới có quà, Kinh doanh có muốn thu hồi quà khi khách xóa bớt món không?</t>
+          <t>Nếu sau này có các gói Combo đặc thù chỉ khi mua Combo mới có suất mua kèm phụ kiện, Kinh doanh có muốn thu hồi quyền mua kèm khi phá Combo không?</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>4. Combo Booster (Bundle Play4 + Dòng khác)</t>
+          <t>4. Combo Booster (Mua kèm khi mua gói Combo thiết bị)</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -1634,24 +1634,24 @@
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>Cộng dồn quyền lợi: 1 Play 4 từ Combo + 2 Play 4 lẻ = Tổng cộng 3 Camera Play 4 → Cấp chính xác 3 suất nhận Charm 0đ.</t>
+          <t>Cộng dồn hạn mức mua kèm: 1 Play 4 từ Combo + 2 Play 4 lẻ = Tổng cộng 3 Camera Play 4 → Cấp chính xác 3 suất mua kèm Charm theo giá ưu đãi.</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>Giao diện hiển thị rõ: 'Bạn có 3 suất mua Charm 0đ (1 từ Combo An Ninh + 2 từ Camera mua lẻ)'.</t>
+          <t>Giao diện hiển thị rõ ràng: 'Bạn có 3 suất mua kèm phụ kiện giá ưu đãi (1 từ Combo An Ninh + 2 từ Camera mua lẻ)'.</t>
         </is>
       </c>
       <c r="H33" s="9" t="inlineStr">
         <is>
-          <t>Có giới hạn số lượng tối đa khi khách vừa mua Combo vừa mua lẻ trong cùng một đơn hàng không?</t>
+          <t>Có áp dụng giới hạn số lượng tối đa phụ kiện mua kèm trên một đơn hàng khi khách vừa mua Combo vừa mua lẻ không?</t>
         </is>
       </c>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>PHẦN 5: 5. DỊCH VỤ BÁM KÈM (GẮN VỚI GÓI CLOUD)</t>
+          <t>PHẦN 5: 5. DỊCH VỤ BÁM KÈM (MUA KÈM GẮN VỚI GÓI CLOUD)</t>
         </is>
       </c>
       <c r="B34" s="5" t="n"/>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>5. Dịch vụ bám kèm (Gắn với gói Cloud)</t>
+          <t>5. Dịch vụ bám kèm (Mua kèm gắn với gói Cloud)</t>
         </is>
       </c>
       <c r="D35" s="12" t="inlineStr">
@@ -1683,22 +1683,22 @@
       </c>
       <c r="E35" s="12" t="inlineStr">
         <is>
-          <t>Chính sách yêu cầu điều kiện kép: Mua Camera Play 4 VÀ đăng ký gói Cloud mới được tặng Charm 0đ.</t>
+          <t>Chính sách quy định điều kiện kép: Mua Camera Play 4 VÀ đăng ký gói Cloud mới được mua kèm Charm giá ưu đãi (0đ).</t>
         </is>
       </c>
       <c r="F35" s="12" t="inlineStr">
         <is>
-          <t>Số lượng quà tính theo số nhỏ nhất (Hàm Min): 3 Camera nhưng chỉ có 1 Cloud → Chỉ được tặng đúng 01 Charm 0đ. 2 Camera còn lại không có Cloud thì không có quà 0đ.</t>
+          <t>Hạn mức mua kèm tính theo số nhỏ nhất (Hàm Min): 3 Camera nhưng chỉ có 1 Cloud → Chỉ có 01 suất mua kèm Charm giá ưu đãi 0đ. 2 Camera còn lại không có Cloud thì không có suất mua kèm giá ưu đãi.</t>
         </is>
       </c>
       <c r="G35" s="12" t="inlineStr">
         <is>
-          <t>Hiển thị lời nhắc: 'Mua thêm 2 gói Cloud để nhận thêm 2 Charm 0đ cho 2 Camera còn lại [Chọn gói Cloud]'.</t>
+          <t>Hiển thị gợi ý: 'Đăng ký thêm 2 gói Cloud để mở thêm 2 suất mua kèm Charm giá ưu đãi cho 2 Camera còn lại [Chọn gói Cloud]'.</t>
         </is>
       </c>
       <c r="H35" s="13" t="inlineStr">
         <is>
-          <t>Đối với 2 Camera không kèm Cloud, Kinh doanh có muốn cho phép khách mua Charm với giá giảm 50% để an ủi không?</t>
+          <t>Đối với 2 Camera không kèm Cloud, Kinh doanh có muốn cho phép khách mua Charm theo chính sách giảm giá 50% không?</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>5. Dịch vụ bám kèm (Gắn với gói Cloud)</t>
+          <t>5. Dịch vụ bám kèm (Mua kèm gắn với gói Cloud)</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
@@ -1723,22 +1723,22 @@
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>Chính sách quy định chỉ gói Cloud từ 6 tháng trở lên mới đủ điều kiện tặng Charm 0đ.</t>
+          <t>Chính sách quy định chỉ gói Cloud từ 6 tháng trở lên mới đủ điều kiện mua kèm Charm giá ưu đãi 0đ.</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
-          <t>Gói Cloud 1 tháng không đủ điều kiện nhận Charm 0đ. Chỉ khi chọn gói Cloud kỳ hạn &gt;= 6 tháng mới mở suất Charm 0đ.</t>
+          <t>Gói Cloud 1 tháng không đủ điều kiện mua kèm Charm giá ưu đãi. Chỉ khi chọn gói Cloud kỳ hạn &gt;= 6 tháng mới mở suất mua kèm Charm giá ưu đãi (0đ).</t>
         </is>
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>Khi khách chọn gói 1 tháng: Hiển thị gợi ý 'Nâng cấp lên gói 6 tháng để nhận ngay Charm Play 4 trị giá 150.000đ hoàn toàn miễn phí'.</t>
+          <t>Khi khách chọn gói 1 tháng: Hiển thị tooltip 'Nâng cấp lên gói 6 tháng để nhận ngay quyền mua kèm Charm Play 4 với giá ưu đãi 0đ'.</t>
         </is>
       </c>
       <c r="H36" s="9" t="inlineStr">
         <is>
-          <t>Kỳ hạn gói Cloud tối thiểu để được tặng Charm 0đ chốt là 6 tháng hay 12 tháng?</t>
+          <t>Kỳ hạn gói Cloud tối thiểu để được hưởng quyền mua kèm Charm giá ưu đãi chốt là 6 tháng hay 12 tháng?</t>
         </is>
       </c>
     </row>
@@ -1753,32 +1753,32 @@
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>5. Dịch vụ bám kèm (Gắn với gói Cloud)</t>
+          <t>5. Dịch vụ bám kèm (Mua kèm gắn với gói Cloud)</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>Hạ gói Cloud trong giỏ: Đang có 1 Cam + Cloud 6T (được 0đ), khách bấm đổi Cloud xuống 1T</t>
+          <t>Hạ gói Cloud trong giỏ: Đang có 1 Cam + Cloud 6T (được giá ưu đãi), khách bấm đổi Cloud xuống 1T</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>Đã có 1 Cam + Cloud 6T + Charm 0đ. Khách đổi thời hạn gói Cloud từ 6T xuống 1T.</t>
+          <t>Đã có 1 Cam + Cloud 6T + Charm giá ưu đãi 0đ. Khách đổi thời hạn gói Cloud từ 6T xuống 1T.</t>
         </is>
       </c>
       <c r="F37" s="12" t="inlineStr">
         <is>
-          <t>Hết điều kiện ưu đãi: Charm 0đ lập tức bị chuyển về giá bán lẻ gốc 150.000đ.</t>
+          <t>Mất điều kiện mua kèm ưu đãi: Charm lập tức bị chuyển về giá bán lẻ niêm yết 150.000đ.</t>
         </is>
       </c>
       <c r="G37" s="12" t="inlineStr">
         <is>
-          <t>Bảng thông báo xác nhận: 'Gói Cloud 1 tháng không đủ điều kiện nhận Charm 0đ. Phụ kiện Charm sẽ được chuyển về giá gốc 150.000đ. Bạn có muốn đổi không?'.</t>
+          <t>Bảng xác nhận: 'Gói Cloud 1 tháng không đủ điều kiện mua kèm Charm giá ưu đãi. Phụ kiện Charm sẽ được tính theo giá bán lẻ 150.000đ. Bạn có muốn đổi không?'.</t>
         </is>
       </c>
       <c r="H37" s="13" t="inlineStr">
         <is>
-          <t>Khi khách hạ gói dịch vụ, Kinh doanh muốn chuyển Charm về giá gốc hay tự động xóa Charm khỏi giỏ hàng?</t>
+          <t>Khi khách hạ gói dịch vụ, Kinh doanh muốn chuyển phụ kiện về giá bán lẻ hay tự động hủy chọn phụ kiện khỏi giỏ hàng?</t>
         </is>
       </c>
     </row>
@@ -1793,39 +1793,39 @@
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>5. Dịch vụ bám kèm (Gắn với gói Cloud)</t>
+          <t>5. Dịch vụ bám kèm (Mua kèm gắn với gói Cloud)</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>Hủy dịch vụ Cloud sau khi đã nhận quà / Hoàn cước Cloud</t>
+          <t>Hủy dịch vụ Cloud sau thanh toán / Hoàn tiền Cloud có phụ kiện mua kèm</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>Khách đã thanh toán đơn gồm Play 4 + Cloud 12T + Charm 0đ. Sau đó khách yêu cầu hủy gói Cloud.</t>
+          <t>Khách đã thanh toán đơn gồm Play 4 + Cloud 12T + Charm mua kèm giá ưu đãi 0đ. Sau đó khách yêu cầu hủy gói Cloud.</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>Khi khách hủy hợp đồng Cloud trước hạn: Số tiền hoàn cước sẽ bị KHẤU TRỪ giá trị niêm yết của Charm (150.000đ). Nếu tiền hoàn nhỏ hơn 150k thì hoàn 0đ.</t>
+          <t>Khi khách hủy hợp đồng Cloud trước hạn: Tiền hoàn cước Cloud sẽ bị KHẤU TRỪ chênh lệch giá niêm yết của Charm (150.000đ - 0đ = 150.000đ) do không còn thỏa điều kiện mua kèm ưu đãi.</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>Nếu khách không đồng ý trừ tiền: Yêu cầu khách hoàn trả lại phụ kiện Charm còn nguyên hộp/nguyên seal về quầy giao dịch FPT.</t>
+          <t>Nếu khách không đồng ý khấu trừ tiền: Yêu cầu khách hoàn trả phụ kiện Charm còn nguyên vẹn/nguyên hộp về quầy giao dịch FPT.</t>
         </is>
       </c>
       <c r="H38" s="9" t="inlineStr">
         <is>
-          <t>Kinh doanh có đồng ý đưa điều khoản ràng buộc này vào hợp đồng cung cấp dịch vụ Cloud để tránh tình trạng trục lợi quà tặng không?</t>
+          <t>Kinh doanh có đồng ý đưa điều khoản ràng buộc khấu trừ phụ kiện mua kèm này vào phụ lục hợp đồng dịch vụ Cloud không?</t>
         </is>
       </c>
     </row>
     <row r="39" ht="28" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>PHẦN 6: 6. GAMIFICATION (MỐC MUA SỈ 3 CAM)</t>
+          <t>PHẦN 6: 6. MUA KÈM PHIÊN BẢN GIỚI HẠN THEO MỐC SỐ LƯỢNG (MỐC 3 CAMERA)</t>
         </is>
       </c>
       <c r="B39" s="5" t="n"/>
@@ -1847,32 +1847,32 @@
       </c>
       <c r="C40" s="12" t="inlineStr">
         <is>
-          <t>6. Gamification (Mốc mua sỉ 3 Cam)</t>
+          <t>6. Mua kèm phiên bản giới hạn theo mốc số lượng (Mốc 3 Camera)</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
-          <t>Đạt mốc thưởng lớn: Đang có 2 Camera, khách bấm tăng lên 3 Camera</t>
+          <t>Đạt mốc số lượng: Đang có 2 Camera, khách bấm tăng lên 3 Camera</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Chính sách: Mua từ 3 Camera trở lên được tặng thêm 01 'Charm Bản Giới Hạn / Limited Edition 0đ'.</t>
+          <t>Chính sách: Khách mua từ 3 Camera trở lên được mở thêm quyền mua kèm 01 'Charm Bản Giới Hạn / Limited Edition' với mức giá ưu đãi đặc biệt (hiện hành: 0đ).</t>
         </is>
       </c>
       <c r="F40" s="12" t="inlineStr">
         <is>
-          <t>Hệ thống tự động mở khóa và thêm ngay 01 Charm Limited Edition (0đ) vào giỏ hàng, đồng thời hạn mức Charm tiêu chuẩn tăng lên 3 chiếc.</t>
+          <t>Hệ thống tự động mở khóa và thêm 01 Charm Limited Edition (giá ưu đãi 0đ) vào giỏ hàng, đồng thời hạn mức mua kèm Charm tiêu chuẩn tăng lên 3 chiếc.</t>
         </is>
       </c>
       <c r="G40" s="12" t="inlineStr">
         <is>
-          <t>Hiển thị thông báo chúc mừng kèm hiệu ứng sinh động trên giỏ hàng để khách hào hứng.</t>
+          <t>Hiển thị thông báo chúc mừng: 'Chúc mừng bạn đã mở khóa quyền mua kèm độc quyền: 01 Charm Limited Edition (0đ)'.</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr">
         <is>
-          <t>Nếu mẫu Charm Limited Edition bị hết hàng trong kho, Kinh doanh muốn thay thế bằng voucher dịch vụ Cloud hay nâng cấp quà tặng khác?</t>
+          <t>Nếu mẫu Charm Limited Edition bị hết hàng trong kho, Kinh doanh muốn thay thế bằng voucher cước Cloud hay nâng cấp sang phụ kiện khác?</t>
         </is>
       </c>
     </row>
@@ -1887,32 +1887,32 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>6. Gamification (Mốc mua sỉ 3 Cam)</t>
+          <t>6. Mua kèm phiên bản giới hạn theo mốc số lượng (Mốc 3 Camera)</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>Hụt mốc thưởng lớn: Đang có 3 Camera + Quà Limited, khách giảm Camera xuống 2</t>
+          <t>Rớt mốc số lượng: Đang có 3 Camera + Charm Limited mua kèm, khách giảm Camera xuống 2</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>Giỏ có 3 Camera + Quà tặng Charm Limited 0đ. Khách giảm số lượng Camera về 2.</t>
+          <t>Giỏ có 3 Camera + Charm Limited mua kèm giá ưu đãi 0đ. Khách giảm số lượng Camera về 2.</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
-          <t>Không còn thỏa điều kiện: Hệ thống tự động thu hồi/xóa quà Charm Limited khỏi giỏ hàng (vì đây là phiên bản quà tặng độc quyền, không bán lẻ).</t>
+          <t>Không còn thỏa điều kiện mốc số lượng: Hệ thống tự động thu hồi/xóa Charm Limited khỏi giỏ hàng (vì đây là phiên bản phụ kiện chỉ mở bán kèm khi đạt mốc số lượng).</t>
         </is>
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
-          <t>Thông báo rõ: 'Số lượng Camera dưới 3, quà tặng Charm Limited Edition đã được tự động gỡ bỏ'.</t>
+          <t>Thông báo rõ: 'Số lượng Camera dưới 3, phụ kiện mua kèm Limited Edition đã được tự động gỡ khỏi giỏ hàng'.</t>
         </is>
       </c>
       <c r="H41" s="9" t="inlineStr">
         <is>
-          <t>Có cần hiển thị cảnh báo trước khi khách bấm giảm không: 'Giảm số lượng sẽ làm mất quà tặng Limited độc quyền'?</t>
+          <t>Có cần hiển thị cảnh báo trước khi khách bấm giảm số lượng: 'Giảm số lượng sẽ làm mất quyền mua kèm phụ kiện Limited Edition'?</t>
         </is>
       </c>
     </row>
@@ -1927,32 +1927,32 @@
       </c>
       <c r="C42" s="12" t="inlineStr">
         <is>
-          <t>6. Gamification (Mốc mua sỉ 3 Cam)</t>
+          <t>6. Mua kèm phiên bản giới hạn theo mốc số lượng (Mốc 3 Camera)</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>Hết quà Limited ngay lúc khách đang thanh toán</t>
+          <t>Hết phụ kiện Limited trong kho ngay lúc khách đang thanh toán</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Khách có 3 Camera + Charm Limited trong giỏ và bấm nút 'Thanh toán'. Kho vừa hết sạch quà Limited.</t>
+          <t>Khách có 3 Camera + Charm Limited trong giỏ và bấm 'Thanh toán'. Kho vừa hết sạch phiên bản Limited.</t>
         </is>
       </c>
       <c r="F42" s="12" t="inlineStr">
         <is>
-          <t>Không chặn đơn hàng Camera của khách: Hệ thống xin lỗi và đề xuất gửi bù quà tặng sau 7 ngày làm việc hoặc cho phép đổi sang quà tặng khác tương đương.</t>
+          <t>Không chặn đơn hàng Camera chính của khách: Hệ thống xin lỗi và cam kết giao bổ sung phụ kiện Limited sau 7 ngày làm việc hoặc cho phép đổi sang phụ kiện khác tương đương.</t>
         </is>
       </c>
       <c r="G42" s="12" t="inlineStr">
         <is>
-          <t>Bảng hỏi: 'Quà tặng Limited vừa hết hàng. Chúng tôi cam kết gửi bù quà miễn phí sau 7 ngày. Bạn có đồng ý tiếp tục đặt hàng không?'.</t>
+          <t>Hộp thoại: 'Phiên bản Charm Limited vừa tạm hết hàng. Chúng tôi cam kết giao bù phụ kiện miễn phí sau 7 ngày. Bạn có đồng ý tiếp tục đặt hàng không?'.</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr">
         <is>
-          <t>Kinh doanh đồng ý giải pháp cam kết gửi bù quà sau để bảo vệ tỷ lệ chốt đơn bán Camera chính hay không?</t>
+          <t>Kinh doanh đồng ý giải pháp cam kết giao bù phụ kiện sau để đảm bảo tỷ lệ chuyển đổi đơn hàng Camera chính hay không?</t>
         </is>
       </c>
     </row>
@@ -1967,39 +1967,39 @@
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>6. Gamification (Mốc mua sỉ 3 Cam)</t>
+          <t>6. Mua kèm phiên bản giới hạn theo mốc số lượng (Mốc 3 Camera)</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>Chống đầu cơ gom hàng quà Limited</t>
+          <t>Chống đầu cơ gom phụ kiện mua kèm Limited Edition</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>Khách hàng hoặc đại lý tạo nhiều đơn hàng liên tục (mỗi đơn 3 Cam) để tích trữ quà Limited.</t>
+          <t>Khách hàng hoặc đại lý tạo nhiều đơn hàng liên tục (mỗi đơn 3 Cam) để gom phụ kiện Limited Edition.</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
         <is>
-          <t>Giới hạn tối đa: Mỗi tài khoản / Số điện thoại / Địa chỉ nhận hàng chỉ được nhận tối đa 02 Charm Limited trong toàn chiến dịch.</t>
+          <t>Giới hạn tối đa: Mỗi tài khoản / Số điện thoại / Địa chỉ nhận hàng chỉ được mua kèm tối đa 02 Charm Limited trong suốt toàn bộ chiến dịch.</t>
         </is>
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>Khi đã nhận đủ 2 quà Limited: Các đơn hàng sau mua 3 Cam chỉ nhận Charm tiêu chuẩn, không tặng thêm bản Limited.</t>
+          <t>Khi đã đạt hạn mức 2 Charm Limited: Các đơn hàng tiếp theo mua 3 Cam vẫn được mua kèm Charm tiêu chuẩn nhưng không mở thêm bản Limited.</t>
         </is>
       </c>
       <c r="H43" s="9" t="inlineStr">
         <is>
-          <t>Kinh doanh muốn siết chặt giới hạn theo Số điện thoại hay Số CCCD/Tài khoản để đảm bảo quà đến tay người dùng thực tế?</t>
+          <t>Kinh doanh muốn kiểm soát hạn mức này theo Số điện thoại hay Số CCCD/Tài khoản để đảm bảo phụ kiện đến tay người dùng thực tế?</t>
         </is>
       </c>
     </row>
     <row r="44" ht="28" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>PHẦN 7: 7. KẾ TOÁN &amp; NỀN TẢNG (DATABASE &amp; VOUCHERS)</t>
+          <t>PHẦN 7: 7. KẾ TOÁN &amp; XUẤT HÓA ĐƠN PHỤ KIỆN MUA KÈM</t>
         </is>
       </c>
       <c r="B44" s="5" t="n"/>
@@ -2021,32 +2021,32 @@
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>7. Kế toán &amp; Nền tảng (Database &amp; Vouchers)</t>
+          <t>7. Kế toán &amp; Xuất hóa đơn phụ kiện mua kèm</t>
         </is>
       </c>
       <c r="D45" s="12" t="inlineStr">
         <is>
-          <t>Xuất hóa đơn điện tử VAT và ghi nhận chứng từ kế toán</t>
+          <t>Xuất hóa đơn điện tử VAT và ghi nhận chứng từ cho phụ kiện bán kèm</t>
         </is>
       </c>
       <c r="E45" s="12" t="inlineStr">
         <is>
-          <t>Đơn hàng thanh toán thành công gồm Camera Play 4 và Charm 0đ.</t>
+          <t>Đơn hàng thanh toán thành công gồm Camera Play 4 và Charm mua kèm giá ưu đãi (0đ).</t>
         </is>
       </c>
       <c r="F45" s="12" t="inlineStr">
         <is>
-          <t>Trên hóa đơn VAT và phiếu bán hàng thể hiện rõ: Charm Play 4 đơn giá 150.000đ - Tiền khuyến mại: -150.000đ - Thành tiền: 0đ theo đúng quy định đăng ký khuyến mại với Sở Công Thương.</t>
+          <t>Trên hóa đơn VAT và phiếu bán hàng thể hiện rõ: Charm Play 4 đơn giá niêm yết 150.000đ - Tiền chiết khấu mua kèm: -150.000đ - Thành tiền: 0đ (hoặc theo mức giá mua kèm thực thu) theo đúng quy định đăng ký chương trình xúc tiến thương mại.</t>
         </is>
       </c>
       <c r="G45" s="12" t="inlineStr">
         <is>
-          <t>Hệ thống ghi nhận chi phí quà tặng vào ngân sách xúc tiến thương mại của bộ phận Marketing/Kinh doanh.</t>
+          <t>Hệ thống ghi nhận chi phí chênh lệch mua kèm vào ngân sách xúc tiến bán hàng của dự án.</t>
         </is>
       </c>
       <c r="H45" s="13" t="inlineStr">
         <is>
-          <t>Mẫu hóa đơn VAT điện tử gửi khách hàng đã được phòng Tài chính - Kế toán duyệt cách thể hiện dòng khuyến mại 0đ này chưa?</t>
+          <t>Mẫu thể hiện hóa đơn VAT cho phụ kiện mua kèm giá 0đ đã được phòng Kế toán duyệt theo quy định thuế chưa?</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>7. Kế toán &amp; Nền tảng (Database &amp; Vouchers)</t>
+          <t>7. Kế toán &amp; Xuất hóa đơn phụ kiện mua kèm</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
@@ -2071,29 +2071,29 @@
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>Khách nhập mã Voucher 'GIAM10 - Giảm 10% tổng đơn' cho giỏ hàng có Camera và phụ kiện.</t>
+          <t>Khách nhập mã Voucher 'GIAM10 - Giảm 10% tổng đơn' cho giỏ hàng có Camera và phụ kiện mua kèm.</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>Voucher giảm % chỉ áp dụng trên giá trị thực thu của Camera và khoản phụ thu (nếu có). Quà tặng 0đ không được tham gia tính giảm thêm.</t>
+          <t>Voucher giảm % chỉ áp dụng trên giá trị thực thu của Camera và khoản phụ thu mua kèm (nếu có). Phụ kiện có giá mua kèm 0đ không được tham gia tính giảm thêm.</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>Hiển thị chi tiết: 'Voucher GIAM10 áp dụng giảm giá trên Camera Play 4 và phụ thu Charm'.</t>
+          <t>Hiển thị chi tiết: 'Voucher GIAM10 áp dụng giảm giá trên Camera Play 4 và phần tiền phụ thu mua kèm'.</t>
         </is>
       </c>
       <c r="H46" s="9" t="inlineStr">
         <is>
-          <t>Chương trình quà tặng Charm có được phép áp dụng chung với các voucher giảm giá/chiết khấu khác trên website không?</t>
+          <t>Chương trình bán kèm phụ kiện giá ưu đãi có được phép áp dụng chung với các voucher giảm giá/chiết khấu khác trên website không?</t>
         </is>
       </c>
     </row>
     <row r="47" ht="28" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>PHẦN 8: 8. QUẢN TRỊ TỒN KHO &amp; CẠNH TRANH GIỎ HÀNG (INVENTORY CONCURRENCY &amp; OOS)</t>
+          <t>PHẦN 8: 8. QUẢN TRỊ TỒN KHO &amp; CẠNH TRANH KHI MUA KÈM PHỤ KIỆN</t>
         </is>
       </c>
       <c r="B47" s="5" t="n"/>
@@ -2115,12 +2115,12 @@
       </c>
       <c r="C48" s="12" t="inlineStr">
         <is>
-          <t>8. Quản trị Tồn kho &amp; Cạnh tranh giỏ hàng (Inventory Concurrency &amp; OOS)</t>
+          <t>8. Quản trị Tồn kho &amp; Cạnh tranh khi mua kèm phụ kiện</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
         <is>
-          <t>Hết hàng tức thời: Mẫu Charm đang chọn bị hết trong kho ngay trước lúc thanh toán</t>
+          <t>Hết hàng tức thời: Mẫu Charm mua kèm bị hết kho ngay trước lúc thanh toán</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -2130,17 +2130,17 @@
       </c>
       <c r="F48" s="12" t="inlineStr">
         <is>
-          <t>Khi bấm 'Thanh toán', nếu mẫu A đã hết, hệ thống nhắc khách đổi sang mẫu Charm khác còn hàng. Không hủy đơn mua Camera của khách.</t>
+          <t>Khi bấm 'Thanh toán', nếu mẫu A đã hết hàng, hệ thống nhắc khách đổi sang mẫu Charm khác còn hàng trong hạn mức mua kèm. Không hủy đơn mua Camera của khách.</t>
         </is>
       </c>
       <c r="G48" s="12" t="inlineStr">
         <is>
-          <t>Mẫu A bị làm mờ, gắn nhãn 'Vừa hết hàng'. Nổi bật nút 'Chọn mẫu khác thay thế'.</t>
+          <t>Mẫu A bị làm mờ, gắn nhãn 'Tạm hết hàng'. Nổi bật nút 'Chọn mẫu phụ kiện khác thay thế'.</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr">
         <is>
-          <t>Nếu tất cả các mẫu Charm đều hết hàng, Kinh doanh có đồng ý phát hành mã voucher trị giá 150k để khách mua phụ kiện ở đợt hàng sau không?</t>
+          <t>Nếu toàn bộ các mẫu phụ kiện Charm đều hết hàng, Kinh doanh có đồng ý cấp mã voucher để khách mua phụ kiện ở đợt hàng sau không?</t>
         </is>
       </c>
     </row>
@@ -2155,32 +2155,32 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>8. Quản trị Tồn kho &amp; Cạnh tranh giỏ hàng (Inventory Concurrency &amp; OOS)</t>
+          <t>8. Quản trị Tồn kho &amp; Cạnh tranh khi mua kèm phụ kiện</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>Tồn kho không đủ số lượng mong muốn: Mua 3 Cam muốn 3 Charm A, nhưng kho chỉ còn 1 cái</t>
+          <t>Tồn kho phụ kiện không đủ số lượng mong muốn: Mua 3 Cam muốn 3 Charm A, nhưng kho chỉ còn 1 cái</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>Kho còn 1 Charm A và nhiều Charm B, C. Khách muốn chọn cả 3 Charm Mẫu A.</t>
+          <t>Kho còn 1 Charm A và nhiều Charm B, C. Khách muốn chọn cả 3 Charm Mẫu A theo giá mua kèm ưu đãi.</t>
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t>Giới hạn số lượng chọn tối đa của mỗi mẫu không vượt quá số lượng tồn kho thực tế. Mẫu A chỉ cho chọn tối đa 1 chiếc.</t>
+          <t>Giới hạn số lượng chọn tối đa của mỗi mẫu phụ kiện không vượt quá số lượng tồn kho thực tế. Mẫu A chỉ cho chọn tối đa 1 chiếc.</t>
         </is>
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>Thông báo: 'Mẫu A chỉ còn 1 sản phẩm. Vui lòng chọn thêm 2 mẫu khác để nhận đủ 3 phần quà tặng'.</t>
+          <t>Thông báo: 'Mẫu A chỉ còn 1 sản phẩm. Vui lòng chọn thêm 2 mẫu phụ kiện khác để tận dụng đủ 3 suất mua kèm ưu đãi'.</t>
         </is>
       </c>
       <c r="H49" s="9" t="inlineStr">
         <is>
-          <t>Kinh doanh có đồng ý hiển thị số lượng tồn kho còn lại của từng mẫu phụ kiện để khách dễ dàng ra quyết định không?</t>
+          <t>Kinh doanh có đồng ý hiển thị số lượng tồn kho còn lại của từng mẫu phụ kiện trên giao diện giỏ hàng không?</t>
         </is>
       </c>
     </row>
@@ -2195,32 +2195,32 @@
       </c>
       <c r="C50" s="12" t="inlineStr">
         <is>
-          <t>8. Quản trị Tồn kho &amp; Cạnh tranh giỏ hàng (Inventory Concurrency &amp; OOS)</t>
+          <t>8. Quản trị Tồn kho &amp; Cạnh tranh khi mua kèm phụ kiện</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
         <is>
-          <t>Để giỏ hàng quá lâu qua đêm (Chương trình khuyến mãi kết thúc)</t>
+          <t>Để giỏ hàng qua đêm (Chính sách giá mua kèm ưu đãi kết thúc hoặc thay đổi)</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>Khách bỏ Camera + Charm vào giỏ lúc đêm. Sáng hôm sau quay lại thanh toán thì chương trình tặng quà đã hết hạn.</t>
+          <t>Khách bỏ Camera + Charm mua kèm giá 0đ vào giỏ lúc đêm. Sáng hôm sau quay lại thanh toán thì chương trình giá ưu đãi đã kết thúc (chuyển sang giá bán lẻ hoặc giá mua kèm mới).</t>
         </is>
       </c>
       <c r="F50" s="12" t="inlineStr">
         <is>
-          <t>Quyền lợi và giá tiền được tính tại thời điểm bấm Đặt hàng. Khi chương trình kết thúc, giỏ hàng tự động cập nhật lại theo giá hiện hành.</t>
+          <t>Giá bán và quyền lợi mua kèm được tính tại thời điểm bấm Đặt hàng (Point of Sale). Khi chính sách kết thúc, giỏ hàng tự động cập nhật lại theo giá hiện hành.</t>
         </is>
       </c>
       <c r="G50" s="12" t="inlineStr">
         <is>
-          <t>Thông báo rõ: 'Chương trình quà tặng Charm 0đ đã kết thúc. Giỏ hàng của bạn đã được cập nhật lại'.</t>
+          <t>Thông báo rõ: 'Chính sách giá mua kèm ưu đãi đã thay đổi. Giỏ hàng của bạn đã được cập nhật lại theo mức giá hiện hành'.</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr">
         <is>
-          <t>Có chính sách ngoại lệ nào gia hạn ưu đãi thêm vài giờ cho khách hàng đã lưu giỏ hàng trước thời điểm hết hạn không?</t>
+          <t>Có chính sách ngoại lệ nào gia hạn mức giá mua kèm cũ thêm một khoảng thời gian cho khách hàng đã lưu giỏ hàng không?</t>
         </is>
       </c>
     </row>
@@ -2264,17 +2264,17 @@
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>Theo cấu hình kinh doanh: Nếu Flash Sale giảm giá quá sâu, sản phẩm Flash Sale KHÔNG áp dụng kèm Charm 0đ.</t>
+          <t>Theo cấu hình kinh doanh: Nếu Flash Sale đã giảm giá quá sâu, sản phẩm Camera Flash Sale KHÔNG áp dụng kèm quyền mua phụ kiện giá ưu đãi 0đ (phụ kiện tính giá bán lẻ bình thường).</t>
         </is>
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>Trang Flash Sale ghi rõ: 'Giá sốc không áp dụng kèm quà tặng Charm 0đ'. Mua theo giá thường vẫn được tặng quà đầy đủ.</t>
+          <t>Trang Flash Sale ghi rõ: 'Giá sốc Flash Sale không áp dụng kèm chính sách mua kèm phụ kiện giá ưu đãi 0đ'.</t>
         </is>
       </c>
       <c r="H52" s="9" t="inlineStr">
         <is>
-          <t>Kinh doanh quyết định: Khi bán giá Flash Sale có kèm quà tặng Charm 0đ không, hay chỉ áp dụng khi bán giá niêm yết?</t>
+          <t>Kinh doanh quyết định: Khi bán Camera giá Flash Sale có kèm quyền mua phụ kiện giá ưu đãi 0đ không, hay chỉ áp dụng khi bán đúng giá niêm yết?</t>
         </is>
       </c>
     </row>
@@ -2294,34 +2294,34 @@
       </c>
       <c r="D53" s="12" t="inlineStr">
         <is>
-          <t>Dùng Điểm thưởng FPT / Xu FPT Loyalty thanh toán phụ thu</t>
+          <t>Dùng Điểm thưởng FPT Loyalty thanh toán khoản phụ thu mua kèm</t>
         </is>
       </c>
       <c r="E53" s="12" t="inlineStr">
         <is>
-          <t>Khách có 50.000 điểm FPT Loyalty, muốn dùng điểm để cấn trừ khoản phụ thu 50k của Charm Premium.</t>
+          <t>Khách có 50.000 điểm FPT Loyalty, muốn dùng điểm để cấn trừ khoản tiền mua kèm 50k của Charm Premium.</t>
         </is>
       </c>
       <c r="F53" s="12" t="inlineStr">
         <is>
-          <t>Cho phép dùng điểm thưởng FPT Loyalty để thanh toán các khoản phụ thu hoặc giá trị thanh toán thực tế (1 điểm = 1 VNĐ).</t>
+          <t>Cho phép dùng điểm thưởng FPT Loyalty để thanh toán các khoản tiền phụ thu mua kèm hoặc tổng giá trị đơn hàng (1 điểm = 1 VNĐ).</t>
         </is>
       </c>
       <c r="G53" s="12" t="inlineStr">
         <is>
-          <t>Mục thanh toán hiển thị: '[x] Dùng 50.000 điểm FPT để thanh toán phụ thu (Số tiền cần trả: 0đ)'.</t>
+          <t>Mục thanh toán hiển thị: '[x] Dùng 50.000 điểm FPT để thanh toán phụ thu mua kèm (Số tiền cần trả: 0đ)'.</t>
         </is>
       </c>
       <c r="H53" s="13" t="inlineStr">
         <is>
-          <t>Kinh doanh có đồng ý cho phép khách dùng điểm thưởng thành viên FPT Loyalty để trừ tiền phụ thu Charm Premium không?</t>
+          <t>Kinh doanh có đồng ý cho phép khách dùng điểm thưởng FPT Loyalty để thanh toán tiền mua kèm phụ kiện không?</t>
         </is>
       </c>
     </row>
     <row r="54" ht="28" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>PHẦN 10: 10. VẬN CHUYỂN &amp; GIAO NHẬN ĐA KHO</t>
+          <t>PHẦN 10: 10. VẬN CHUYỂN &amp; GIAO NHẬN ĐA KHO CHO PHỤ KIỆN MUA KÈM</t>
         </is>
       </c>
       <c r="B54" s="5" t="n"/>
@@ -2343,12 +2343,12 @@
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>10. Vận chuyển &amp; Giao nhận Đa kho</t>
+          <t>10. Vận chuyển &amp; Giao nhận Đa kho cho phụ kiện mua kèm</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>Lệch kho hàng: Kho gần khách có Camera nhưng hết Charm (Charm ở kho khác)</t>
+          <t>Lệch kho hàng: Kho gần khách có Camera nhưng hết phụ kiện mua kèm (Phụ kiện ở kho khác)</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -2358,12 +2358,12 @@
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t>Hệ thống tự động tối ưu: Điều chuyển Charm về để giao chung 1 lần; HOẶC Tách làm 2 kiện giao riêng mà KHÔNG thu thêm bất kỳ phí vận chuyển nào của khách.</t>
+          <t>Hệ thống tối ưu điều phối: Điều chuyển Charm về để gom giao chung 1 lần; HOẶC Tách làm 2 kiện giao riêng mà KHÔNG thu thêm bất kỳ chi phí vận chuyển nào của khách đối với kiện phụ kiện mua kèm.</t>
         </is>
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t>Màn hình đặt hàng thông báo: 'Đơn hàng được chia làm 2 kiện do phụ kiện chuyển từ kho đặc biệt. Miễn phí vận chuyển cho phụ kiện quà tặng'.</t>
+          <t>Màn hình đặt hàng thông báo: 'Đơn hàng được chia làm 2 kiện do phụ kiện mua kèm chuyển từ kho khác. Miễn phí vận chuyển cho kiện phụ kiện mua kèm'.</t>
         </is>
       </c>
       <c r="H55" s="9" t="inlineStr">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C56" s="12" t="inlineStr">
         <is>
-          <t>10. Vận chuyển &amp; Giao nhận Đa kho</t>
+          <t>10. Vận chuyển &amp; Giao nhận Đa kho cho phụ kiện mua kèm</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
@@ -2393,29 +2393,29 @@
       </c>
       <c r="E56" s="12" t="inlineStr">
         <is>
-          <t>Khách đặt hàng trên web và chọn đến Shop FPT nhận hàng.</t>
+          <t>Khách đặt mua Camera kèm phụ kiện trên web và chọn đến Shop FPT nhận hàng.</t>
         </is>
       </c>
       <c r="F56" s="12" t="inlineStr">
         <is>
-          <t>Kiểm tra tồn kho tại Shop: Nếu Shop có sẵn Camera nhưng thiếu Charm, hệ thống báo thời gian điều chuyển Charm về Shop trước khi khách ra lấy.</t>
+          <t>Kiểm tra tồn kho tại Shop: Nếu Shop có sẵn Camera nhưng thiếu phụ kiện mua kèm, hệ thống thông báo thời gian điều chuyển phụ kiện về Shop trước khi khách ra lấy.</t>
         </is>
       </c>
       <c r="G56" s="12" t="inlineStr">
         <is>
-          <t>Thông báo: 'Cửa hàng có sẵn Camera. Phụ kiện Charm dự kiến có mặt tại Shop sau 24h. Chúng tôi sẽ gửi tin nhắn SMS khi trọn bộ sẵn sàng'.</t>
+          <t>Thông báo: 'Cửa hàng có sẵn Camera. Phụ kiện mua kèm dự kiến có mặt tại Shop sau 24h. Chúng tôi sẽ gửi tin nhắn SMS khi trọn bộ sẵn sàng'.</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr">
         <is>
-          <t>Khách có được phép lấy Camera trước tại quầy, còn quà tặng Charm sẽ gửi chuyển phát về tận nhà miễn phí sau không?</t>
+          <t>Khách có được phép nhận Camera trước tại quầy, còn phụ kiện mua kèm sẽ gửi chuyển phát về tận nhà miễn phí sau không?</t>
         </is>
       </c>
     </row>
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>PHẦN 11: 11. CỔNG THANH TOÁN &amp; TRẠNG THÁI ĐƠN HÀNG</t>
+          <t>PHẦN 11: 11. CỔNG THANH TOÁN &amp; TRẠNG THÁI ĐƠN HÀNG MUA KÈM</t>
         </is>
       </c>
       <c r="B57" s="5" t="n"/>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>11. Cổng thanh toán &amp; Trạng thái đơn hàng</t>
+          <t>11. Cổng thanh toán &amp; Trạng thái đơn hàng mua kèm</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
@@ -2447,12 +2447,12 @@
       </c>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t>Khách chọn thanh toán qua VNPAY/MoMo nhưng để quá 15 phút không hoàn tất.</t>
+          <t>Khách chọn thanh toán qua VNPAY/MoMo cho đơn gồm Camera và phụ kiện mua kèm nhưng để quá 15 phút không thanh toán.</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>Hạn mức ưu đãi và tồn kho Charm được tạm giữ trong 15 phút. Sau 15 phút không thanh toán, đơn tự hủy và giải phóng tồn kho cho khách khác mua.</t>
+          <t>Hạn mức mua kèm ưu đãi và tồn kho phụ kiện được tạm giữ trong 15 phút. Sau 15 phút không hoàn tất, đơn tự hủy và giải phóng tồn kho cho khách khác.</t>
         </is>
       </c>
       <c r="G58" s="8" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="H58" s="9" t="inlineStr">
         <is>
-          <t>Thời gian chờ thanh toán trực tuyến đối với đơn hàng có quà tặng nên là 15 phút hay 30 phút?</t>
+          <t>Thời gian giữ chỗ tồn kho và hạn mức mua kèm khi thanh toán trực tuyến nên là 15 phút hay 30 phút?</t>
         </is>
       </c>
     </row>
@@ -2477,39 +2477,39 @@
       </c>
       <c r="C59" s="12" t="inlineStr">
         <is>
-          <t>11. Cổng thanh toán &amp; Trạng thái đơn hàng</t>
+          <t>11. Cổng thanh toán &amp; Trạng thái đơn hàng mua kèm</t>
         </is>
       </c>
       <c r="D59" s="12" t="inlineStr">
         <is>
-          <t>Khách hủy đơn hàng thanh toán khi nhận hàng (COD) trước khi xuất kho</t>
+          <t>Khách hủy đơn hàng COD trước khi xuất kho</t>
         </is>
       </c>
       <c r="E59" s="12" t="inlineStr">
         <is>
-          <t>Đơn hàng COD đang ở trạng thái 'Chờ xác nhận'. Khách bấm 'Hủy đơn hàng' trên web.</t>
+          <t>Đơn hàng COD gồm Camera và phụ kiện mua kèm đang ở trạng thái 'Chờ xác nhận'. Khách bấm 'Hủy đơn hàng' trên web.</t>
         </is>
       </c>
       <c r="F59" s="12" t="inlineStr">
         <is>
-          <t>Cho phép khách hủy đơn ngay lập tức nếu hàng chưa bàn giao cho shipper. Toàn bộ hạn mức mua quà và tồn kho phụ kiện được hoàn trả về hệ thống.</t>
+          <t>Cho phép khách hủy đơn ngay lập tức nếu hàng chưa bàn giao cho shipper. Toàn bộ hạn mức mua kèm ưu đãi và tồn kho phụ kiện được hoàn trả về hệ thống.</t>
         </is>
       </c>
       <c r="G59" s="12" t="inlineStr">
         <is>
-          <t>Hiển thị danh sách lý do hủy đơn để khách phản hồi (Đổi ý, chọn nhầm mẫu Charm, muốn mua thêm Camera).</t>
+          <t>Hiển thị danh sách lý do hủy đơn để khách phản hồi (Đổi ý, chọn nhầm mẫu phụ kiện, muốn đổi địa chỉ).</t>
         </is>
       </c>
       <c r="H59" s="13" t="inlineStr">
         <is>
-          <t>Sau khi khách tự hủy đơn có quà tặng, có cần gửi tin nhắn kèm ưu đãi giữ chân khách hàng quay lại mua không?</t>
+          <t>Sau khi khách tự hủy đơn, có cần gửi tin nhắn kèm ưu đãi giữ chân khách hàng quay lại mua không?</t>
         </is>
       </c>
     </row>
     <row r="60" ht="28" customHeight="1">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>PHẦN 12: 12. ĐỔI TRẢ TỪNG PHẦN &amp; BẢO HÀNH (RMA &amp; WARRANTY)</t>
+          <t>PHẦN 12: 12. ĐỔI TRẢ TỪNG PHẦN &amp; BẢO HÀNH PHỤ KIỆN MUA KÈM (RMA &amp; WARRANTY)</t>
         </is>
       </c>
       <c r="B60" s="5" t="n"/>
@@ -2531,7 +2531,7 @@
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>12. Đổi trả từng phần &amp; Bảo hành (RMA &amp; Warranty)</t>
+          <t>12. Đổi trả từng phần &amp; Bảo hành phụ kiện mua kèm (RMA &amp; Warranty)</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
@@ -2541,22 +2541,22 @@
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>Camera bị lỗi phần cứng trong thời gian bảo hành chính hãng.</t>
+          <t>Camera chính bị lỗi phần cứng trong thời gian bảo hành chính hãng.</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
-          <t>Kỹ thuật viên / Cửa hàng đổi mới 01 Camera Play 4 tương đương cho khách. Khách KHÔNG phải nộp lại phụ kiện Charm đã tặng.</t>
+          <t>Kỹ thuật viên / Cửa hàng đổi mới 01 Camera Play 4 tương đương cho khách. Khách KHÔNG phải nộp lại phụ kiện Charm đã mua kèm.</t>
         </is>
       </c>
       <c r="G61" s="8" t="inlineStr">
         <is>
-          <t>Phiếu bảo hành ghi rõ: 'Đổi mới Camera Play 4 - Không thu hồi phụ kiện khuyến mại Charm'.</t>
+          <t>Phiếu bảo hành ghi rõ: 'Đổi mới Camera Play 4 - Khách giữ nguyên phụ kiện mua kèm Charm'.</t>
         </is>
       </c>
       <c r="H61" s="9" t="inlineStr">
         <is>
-          <t>Nếu phụ kiện Charm bị lỗi sản xuất (ví dụ gãy khớp nối), Kinh doanh có chính sách đổi mới phụ kiện trong vòng bao nhiêu ngày?</t>
+          <t>Nếu bản thân phụ kiện Charm bị lỗi sản xuất (ví dụ gãy khớp nối), Kinh doanh có chính sách bảo hành 1 đổi 1 phụ kiện trong bao nhiêu ngày?</t>
         </is>
       </c>
     </row>
@@ -2571,39 +2571,39 @@
       </c>
       <c r="C62" s="12" t="inlineStr">
         <is>
-          <t>12. Đổi trả từng phần &amp; Bảo hành (RMA &amp; Warranty)</t>
+          <t>12. Đổi trả từng phần &amp; Bảo hành phụ kiện mua kèm (RMA &amp; Warranty)</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>Khách trả hàng Camera Play 4 để lấy lại tiền mặt</t>
+          <t>Khách trả Camera Play 4 để lấy lại tiền mặt (Chính sách trả hàng có phụ kiện mua kèm)</t>
         </is>
       </c>
       <c r="E62" s="12" t="inlineStr">
         <is>
-          <t>Đơn hàng gồm 1 Cam (800k) + 1 Charm 0đ (giá niêm yết 150k). Sau 3 ngày khách yêu cầu trả Camera đòi lại tiền.</t>
+          <t>Đơn hàng gồm 1 Cam (800k) + 1 Charm mua kèm giá ưu đãi 0đ (giá niêm yết 150k). Sau 3 ngày khách yêu cầu trả Camera đòi lại tiền.</t>
         </is>
       </c>
       <c r="F62" s="12" t="inlineStr">
         <is>
-          <t>Khách phải hoàn trả lại Camera kèm phụ kiện Charm còn nguyên seal/hộp. Nếu Charm đã bị mất hoặc hư hỏng, khấu trừ giá trị niêm yết của Charm (150.000đ) vào số tiền hoàn của Camera (Khách nhận lại 650.000đ).</t>
+          <t>Khách trả Camera chính thì phụ kiện mua kèm không còn thỏa điều kiện hưởng giá ưu đãi: Khách phải hoàn trả lại Camera kèm phụ kiện Charm còn nguyên vẹn. Nếu khách giữ lại Charm hoặc Charm đã hư hỏng, hệ thống sẽ KHẤU TRỪ giá bán lẻ niêm yết của Charm (150.000đ) vào số tiền hoàn lại của Camera (Khách chỉ nhận lại 650.000đ).</t>
         </is>
       </c>
       <c r="G62" s="12" t="inlineStr">
         <is>
-          <t>Charm Premium phụ thu 50k: Nếu chỉ trả Camera giữ Charm, hoàn tiền = 800k - (200k - 50k) = 650k.</t>
+          <t>Trường hợp Charm Premium phụ thu 50k: Nếu chỉ trả Camera giữ Charm Premium, hoàn tiền = 800k - (200k - 50k) = 650.000đ.</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr">
         <is>
-          <t>Kinh doanh chọn phương án nào: (A) Khấu trừ theo giá niêm yết 150k; (B) Khấu trừ theo giá vốn nhập hàng; hay (C) Bắt buộc trả đủ cả bộ mới cho hoàn tiền?</t>
+          <t>Kinh doanh chọn phương án xử lý phụ kiện mua kèm khi trả hàng: (A) Khấu trừ theo giá bán lẻ niêm yết; (B) Khấu trừ theo giá vốn; hay (C) Bắt buộc trả đủ trọn bộ mới cho hoàn tiền?</t>
         </is>
       </c>
     </row>
     <row r="63" ht="28" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>PHẦN 13: 13. TRẢI NGHIỆM KHÁCH VÃNG LAI &amp; ĐĂNG NHẬP TÀI KHOẢN</t>
+          <t>PHẦN 13: 13. TRẢI NGHIỆM KHÁCH VÃNG LAI &amp; ĐĂNG NHẬP TÀI KHOẢN KHI MUA KÈM</t>
         </is>
       </c>
       <c r="B63" s="5" t="n"/>
@@ -2625,32 +2625,32 @@
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t>13. Trải nghiệm Khách vãng lai &amp; Đăng nhập tài khoản</t>
+          <t>13. Trải nghiệm Khách vãng lai &amp; Đăng nhập tài khoản khi mua kèm</t>
         </is>
       </c>
       <c r="D64" s="8" t="inlineStr">
         <is>
-          <t>Khách vãng lai (chưa đăng nhập) chọn hàng rồi mới bấm Đăng nhập</t>
+          <t>Khách vãng lai chọn Camera và phụ kiện mua kèm rồi mới bấm Đăng nhập</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t>Khách chưa đăng nhập chọn 1 Cam + 1 Charm A (0đ). Sau đó bấm Đăng nhập. Tài khoản đã có sẵn 1 Cam từ trước.</t>
+          <t>Khách chưa đăng nhập chọn 1 Cam + 1 Charm A (giá mua kèm ưu đãi). Sau đó bấm Đăng nhập. Tài khoản đã có sẵn 1 Cam từ trước.</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t>Hợp nhất giỏ hàng thông minh: Tổng số Camera = 1 (vãng lai) + 1 (tài khoản) = 2 Camera. Suất quà Charm 0đ tự động nâng lên 2. Giữ nguyên Charm A và mở thêm 1 ô quà thứ 2.</t>
+          <t>Hợp nhất giỏ hàng thông minh: Tổng số Camera = 1 (vãng lai) + 1 (tài khoản) = 2 Camera. Hạn mức mua kèm phụ kiện giá ưu đãi tự động nâng lên 2. Giữ nguyên Charm A và mở thêm 1 suất mua kèm ưu đãi thứ 2.</t>
         </is>
       </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>Thông báo: 'Giỏ hàng đã được đồng bộ. Bạn hiện có 2 Camera và 2 suất nhận Charm 0đ! [Chọn thêm quà]'.</t>
+          <t>Thông báo: 'Giỏ hàng đã được đồng bộ. Bạn hiện có 2 Camera và 2 suất mua kèm phụ kiện giá ưu đãi! [Chọn thêm phụ kiện]'.</t>
         </is>
       </c>
       <c r="H64" s="9" t="inlineStr">
         <is>
-          <t>Nếu giỏ hàng cũ trên tài khoản đã có sẵn Charm B, Kinh doanh muốn hệ thống tự gộp thành (Charm A + Charm B = 2 quà 0đ) luôn không?</t>
+          <t>Nếu giỏ hàng cũ trên tài khoản đã có sẵn Charm B, Kinh doanh muốn hệ thống tự gộp thành (Charm A + Charm B = 2 phụ kiện mua kèm ưu đãi) luôn không?</t>
         </is>
       </c>
     </row>
@@ -2665,32 +2665,32 @@
       </c>
       <c r="C65" s="12" t="inlineStr">
         <is>
-          <t>13. Trải nghiệm Khách vãng lai &amp; Đăng nhập tài khoản</t>
+          <t>13. Trải nghiệm Khách vãng lai &amp; Đăng nhập tài khoản khi mua kèm</t>
         </is>
       </c>
       <c r="D65" s="12" t="inlineStr">
         <is>
-          <t>Khách đăng xuất tài khoản khi đang có giỏ hàng khuyến mãi</t>
+          <t>Khách đăng xuất tài khoản khi đang có giỏ hàng phụ kiện mua kèm</t>
         </is>
       </c>
       <c r="E65" s="12" t="inlineStr">
         <is>
-          <t>Khách đang có giỏ hàng khuyến mãi Camera + Charm, sau đó bấm 'Đăng xuất'.</t>
+          <t>Khách đang có giỏ hàng Camera + phụ kiện mua kèm giá ưu đãi, sau đó bấm 'Đăng xuất'.</t>
         </is>
       </c>
       <c r="F65" s="12" t="inlineStr">
         <is>
-          <t>Giỏ hàng khuyến mãi của tài khoản được lưu an toàn trên hệ thống. Trình duyệt công cộng được làm sạch giỏ hàng để bảo mật.</t>
+          <t>Giỏ hàng cùng các điều kiện mua kèm ưu đãi của tài khoản được lưu an toàn trên hệ thống. Trình duyệt công cộng được làm sạch giỏ hàng để bảo mật.</t>
         </is>
       </c>
       <c r="G65" s="12" t="inlineStr">
         <is>
-          <t>Khi đăng nhập lại từ bất kỳ thiết bị nào, giỏ hàng cùng các quyền lợi ưu đãi quà tặng được phục hồi nguyên vẹn.</t>
+          <t>Khi đăng nhập lại từ bất kỳ thiết bị nào, giỏ hàng cùng các quyền lợi mua kèm ưu đãi được phục hồi nguyên vẹn.</t>
         </is>
       </c>
       <c r="H65" s="13" t="inlineStr">
         <is>
-          <t>Giỏ hàng khuyến mãi lưu trên tài khoản khách hàng nên được lưu giữ tối đa bao nhiêu ngày trước khi tự động làm mới?</t>
+          <t>Giỏ hàng mua kèm phụ kiện lưu trên tài khoản khách hàng nên được lưu giữ tối đa bao nhiêu ngày trước khi tự động làm mới?</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(cart-spec): bo sung 4 module use case luong ban moi tren website (PDP, Mini-cart, Checkout, Post-purchase)
</commit_message>
<xml_diff>
--- a/thuyttdoc/Kich_Ban_Ky_Thuat_Play4_Charm.xlsx
+++ b/thuyttdoc/Kich_Ban_Ky_Thuat_Play4_Charm.xlsx
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2694,16 +2694,436 @@
         </is>
       </c>
     </row>
+    <row r="66" ht="28" customHeight="1">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>PHẦN 14: 14. MUA NHANH (BUY NOW) &amp; KHỐI BÁN KÈM TRÊN TRANG SẢN PHẨM (PDP)</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="n"/>
+      <c r="C66" s="5" t="n"/>
+      <c r="D66" s="5" t="n"/>
+      <c r="E66" s="5" t="n"/>
+      <c r="F66" s="5" t="n"/>
+      <c r="G66" s="5" t="n"/>
+      <c r="H66" s="5" t="n"/>
+    </row>
+    <row r="67" ht="70" customHeight="1">
+      <c r="A67" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>BR-01</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>14. Mua Nhanh (Buy Now) &amp; Khối Bán Kèm trên Trang Sản Phẩm (PDP)</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Khách bấm nút 'MUA NGAY' (Express Checkout) trên trang Camera Play 4</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>Khách đang xem trang chi tiết Camera Play 4 và bấm nút 'MUA NGAY' để đi thẳng đến bước thanh toán.</t>
+        </is>
+      </c>
+      <c r="F67" s="8" t="inlineStr">
+        <is>
+          <t>Bật Pop-up nhanh (Quick Add-on Modal) trước khi chuyển hướng: 'Bạn được tặng 01 suất mua kèm Charm ưu đãi 0đ. Bạn có muốn nhận ngay không?' kèm danh sách mẫu Charm còn hàng và 2 nút: [Nhận phụ kiện 0đ &amp; Thanh toán] hoặc [Bỏ qua &amp; Đến thanh toán].</t>
+        </is>
+      </c>
+      <c r="G67" s="8" t="inlineStr">
+        <is>
+          <t>Nếu khách bấm 'Bỏ qua': Hệ thống chuyển thẳng sang Checkout chỉ với Camera Play 4, không ép buộc chọn phụ kiện.</t>
+        </is>
+      </c>
+      <c r="H67" s="9" t="inlineStr">
+        <is>
+          <t>Kinh doanh muốn bật Pop-up chọn nhanh phụ kiện khi bấm 'Mua ngay' hay chuyển thẳng sang Checkout rồi nhắc chọn phụ kiện tại trang Checkout?</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="70" customHeight="1">
+      <c r="A68" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="B68" s="11" t="inlineStr">
+        <is>
+          <t>BR-02</t>
+        </is>
+      </c>
+      <c r="C68" s="12" t="inlineStr">
+        <is>
+          <t>14. Mua Nhanh (Buy Now) &amp; Khối Bán Kèm trên Trang Sản Phẩm (PDP)</t>
+        </is>
+      </c>
+      <c r="D68" s="12" t="inlineStr">
+        <is>
+          <t>Khối hiển thị mua kèm (Attached Deal Widget) trên trang chi tiết sản phẩm</t>
+        </is>
+      </c>
+      <c r="E68" s="12" t="inlineStr">
+        <is>
+          <t>Khách xem Camera Play 4, bên dưới có khối 'Ưu đãi mua kèm phụ kiện độc quyền'.</t>
+        </is>
+      </c>
+      <c r="F68" s="12" t="inlineStr">
+        <is>
+          <t>Mặc định KHÔNG tick sẵn phụ kiện để tránh khách không có nhu cầu hoặc chọn nhầm màu. Khách tick chọn mẫu Charm mong muốn thì nút 'Thêm vào giỏ' sẽ tự động gom cả Camera và Charm vào giỏ hàng trong 1 lần bấm.</t>
+        </is>
+      </c>
+      <c r="G68" s="12" t="inlineStr">
+        <is>
+          <t>Nếu khách tăng số lượng Camera lên 2 tại PDP: Hiển thị tooltip 'Bạn được mua kèm 2 Charm giá ưu đãi! Bạn có thể chọn thêm mẫu khác trong giỏ hàng'.</t>
+        </is>
+      </c>
+      <c r="H68" s="13" t="inlineStr">
+        <is>
+          <t>Kinh doanh muốn mặc định tick sẵn 1 mẫu phụ kiện hay để trống cho khách tự chủ động chọn?</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="70" customHeight="1">
+      <c r="A69" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>BR-03</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>14. Mua Nhanh (Buy Now) &amp; Khối Bán Kèm trên Trang Sản Phẩm (PDP)</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>Biến thể phụ kiện mua kèm bị Hết hàng (Out of Stock) tại trang sản phẩm</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>Charm Mẫu A (Màu Hồng) hết hàng trong kho, các mẫu B và C vẫn còn hàng.</t>
+        </is>
+      </c>
+      <c r="F69" s="8" t="inlineStr">
+        <is>
+          <t>Tại khối mua kèm trên PDP: Mẫu A hiển thị dưới dạng làm mờ (Grey-out), gắn nhãn 'Tạm hết hàng' và khóa không cho tick chọn. Các mẫu còn hàng hiển thị bình thường kèm nhãn 'Giá ưu đãi 0đ'.</t>
+        </is>
+      </c>
+      <c r="G69" s="8" t="inlineStr">
+        <is>
+          <t>Nếu tất cả các mẫu Charm đều hết hàng: Khối mua kèm tự động ẩn khỏi trang PDP để tránh gây bức xúc cho khách hàng.</t>
+        </is>
+      </c>
+      <c r="H69" s="9" t="inlineStr">
+        <is>
+          <t>Khi một mẫu phụ kiện hết hàng, Kinh doanh muốn làm mờ gắn nhãn 'Tạm hết' hay ẩn hoàn toàn mẫu đó khỏi trang sản phẩm?</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="28" customHeight="1">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>PHẦN 15: 15. THAO TÁC BÁN KÈM TRÊN GIỎ HÀNG TRƯỢT (MINI-CART / DRAWER CART)</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="n"/>
+      <c r="C70" s="5" t="n"/>
+      <c r="D70" s="5" t="n"/>
+      <c r="E70" s="5" t="n"/>
+      <c r="F70" s="5" t="n"/>
+      <c r="G70" s="5" t="n"/>
+      <c r="H70" s="5" t="n"/>
+    </row>
+    <row r="71" ht="70" customHeight="1">
+      <c r="A71" s="10" t="n">
+        <v>52</v>
+      </c>
+      <c r="B71" s="11" t="inlineStr">
+        <is>
+          <t>BR-01</t>
+        </is>
+      </c>
+      <c r="C71" s="12" t="inlineStr">
+        <is>
+          <t>15. Thao tác Bán kèm trên Giỏ Hàng Trượt (Mini-Cart / Drawer Cart)</t>
+        </is>
+      </c>
+      <c r="D71" s="12" t="inlineStr">
+        <is>
+          <t>Đổi mẫu phụ kiện mua kèm trực tiếp trên ngăn kéo Mini-Cart</t>
+        </is>
+      </c>
+      <c r="E71" s="12" t="inlineStr">
+        <is>
+          <t>Khách thêm Camera + 1 Charm A vào giỏ. Mini-cart bên phải màn hình trượt ra.</t>
+        </is>
+      </c>
+      <c r="F71" s="12" t="inlineStr">
+        <is>
+          <t>Tại dòng Charm A trên Mini-cart, hiển thị nút bấm nhỏ '[Đổi mẫu]'. Khi khách bấm, mở danh sách popover các mẫu Charm còn hàng để khách chuyển đổi sang Charm B ngay trên Mini-cart mà không cần chuyển trang.</t>
+        </is>
+      </c>
+      <c r="G71" s="12" t="inlineStr">
+        <is>
+          <t>Nếu khách chọn đổi sang Charm Premium (+50k): Subtotal của Mini-cart tự động cập nhật cộng thêm 50.000đ ngay lập tức.</t>
+        </is>
+      </c>
+      <c r="H71" s="13" t="inlineStr">
+        <is>
+          <t>Kinh doanh có đồng ý cho khách đổi mẫu phụ kiện ngay trên Mini-cart không hay bắt buộc phải vào trang Giỏ hàng chi tiết (/cart)?</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="70" customHeight="1">
+      <c r="A72" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>BR-02</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>15. Thao tác Bán kèm trên Giỏ Hàng Trượt (Mini-Cart / Drawer Cart)</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>Tăng số lượng Camera trực tiếp trên Mini-Cart</t>
+        </is>
+      </c>
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>Mini-cart đang có 1 Camera + 1 Charm A (0đ). Khách bấm nút [+] tăng Camera lên 2.</t>
+        </is>
+      </c>
+      <c r="F72" s="8" t="inlineStr">
+        <is>
+          <t>Hạn mức ưu đãi tăng lên 2. Giữ nguyên 1 Charm A đã chọn, đồng thời bên dưới xuất hiện 1 dòng slot trống nổi bật: '+ Thêm 1 Charm ưu đãi 0đ [Chọn ngay]'.</t>
+        </is>
+      </c>
+      <c r="G72" s="8" t="inlineStr">
+        <is>
+          <t>Nếu khách bấm 'Thanh toán' mà chưa chọn slot thứ 2: Đơn hàng vẫn tiếp tục bình thường với 2 Camera + 1 Charm A.</t>
+        </is>
+      </c>
+      <c r="H72" s="9" t="inlineStr">
+        <is>
+          <t>Khi tăng Camera trên Mini-cart, Kinh doanh muốn hệ thống tự động nhân đôi mẫu Charm hiện tại hay mở slot trống để khách tự chọn?</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="28" customHeight="1">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>PHẦN 16: 16. RÀNG BUỘC KHUYẾN MÃI &amp; KHO TẠI TRANG THANH TOÁN (CHECKOUT)</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="n"/>
+      <c r="C73" s="5" t="n"/>
+      <c r="D73" s="5" t="n"/>
+      <c r="E73" s="5" t="n"/>
+      <c r="F73" s="5" t="n"/>
+      <c r="G73" s="5" t="n"/>
+      <c r="H73" s="5" t="n"/>
+    </row>
+    <row r="74" ht="70" customHeight="1">
+      <c r="A74" s="10" t="n">
+        <v>54</v>
+      </c>
+      <c r="B74" s="11" t="inlineStr">
+        <is>
+          <t>BR-01</t>
+        </is>
+      </c>
+      <c r="C74" s="12" t="inlineStr">
+        <is>
+          <t>16. Ràng buộc Khuyến mãi &amp; Kho tại Trang Thanh Toán (Checkout)</t>
+        </is>
+      </c>
+      <c r="D74" s="12" t="inlineStr">
+        <is>
+          <t>Lời nhắc cuối (Last Reminder) tại Trang Thanh toán khi chưa chọn phụ kiện</t>
+        </is>
+      </c>
+      <c r="E74" s="12" t="inlineStr">
+        <is>
+          <t>Khách mua Camera Play 4 nhưng chưa chọn phụ kiện mua kèm nào và đã đến trang Checkout điền địa chỉ.</t>
+        </is>
+      </c>
+      <c r="F74" s="12" t="inlineStr">
+        <is>
+          <t>Ngay phía trên nút 'Đặt hàng', hiển thị Banner ưu đãi 1 chạm: 'Bạn đang bỏ lỡ 01 Charm Play 4 giá ưu đãi 0đ! [Nhận Charm ngay]'. Khách click chọn mẫu là hệ thống tự add vào đơn ngay tại Checkout mà không reload trang.</t>
+        </is>
+      </c>
+      <c r="G74" s="12" t="inlineStr">
+        <is>
+          <t>Khách có quyền bấm 'Bỏ qua' hoặc nhấn thẳng nút 'Đặt hàng' nếu không có nhu cầu.</t>
+        </is>
+      </c>
+      <c r="H74" s="13" t="inlineStr">
+        <is>
+          <t>Có cần hiển thị Banner nhắc nhận phụ kiện 0đ ngay tại bước Thanh toán cuối cùng để tối ưu tỷ lệ gắn kèm sản phẩm không?</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="70" customHeight="1">
+      <c r="A75" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>BR-02</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>16. Ràng buộc Khuyến mãi &amp; Kho tại Trang Thanh Toán (Checkout)</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>Khách nhập Mã giảm giá (Coupon Code) xung đột với suất mua kèm</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>Khách có Camera và Charm (0đ) trong đơn, khách nhập mã voucher toàn sàn (VD: Mã GIAM50K cho đơn từ 1.000.000đ).</t>
+        </is>
+      </c>
+      <c r="F75" s="8" t="inlineStr">
+        <is>
+          <t>Giá trị của Charm 0đ KHÔNG được tính vào điều kiện giá trị đơn hàng tối thiểu (Min Basket Size) để kích hoạt voucher. Voucher chỉ giảm trên số tiền thực thu của Camera và phần phụ thu mua kèm (nếu có).</t>
+        </is>
+      </c>
+      <c r="G75" s="8" t="inlineStr">
+        <is>
+          <t>Nếu khách nhập voucher chuyên biệt dành cho phụ kiện: Hệ thống áp dụng quy tắc ưu đãi tốt nhất, không cộng dồn hai mức giảm giá cho cùng 1 món.</t>
+        </is>
+      </c>
+      <c r="H75" s="9" t="inlineStr">
+        <is>
+          <t>Phụ kiện mua kèm giá 0đ có được tính vào tổng giá trị đơn hàng để xét điều kiện áp dụng mã voucher toàn sàn không?</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="70" customHeight="1">
+      <c r="A76" s="10" t="n">
+        <v>56</v>
+      </c>
+      <c r="B76" s="11" t="inlineStr">
+        <is>
+          <t>BR-03</t>
+        </is>
+      </c>
+      <c r="C76" s="12" t="inlineStr">
+        <is>
+          <t>16. Ràng buộc Khuyến mãi &amp; Kho tại Trang Thanh Toán (Checkout)</t>
+        </is>
+      </c>
+      <c r="D76" s="12" t="inlineStr">
+        <is>
+          <t>Khách đổi Địa chỉ nhận hàng tại Checkout dẫn đến Lệch kho tồn phụ kiện</t>
+        </is>
+      </c>
+      <c r="E76" s="12" t="inlineStr">
+        <is>
+          <t>Khách đổi địa chỉ giao hàng từ Hà Nội (kho còn Charm) sang tỉnh khác (kho tỉnh hết Charm, chỉ còn kho trung tâm).</t>
+        </is>
+      </c>
+      <c r="F76" s="12" t="inlineStr">
+        <is>
+          <t>Không tự ý gỡ Charm của khách: Hệ thống hiển thị thông báo thời gian giao hàng: 'Phụ kiện mua kèm sẽ được điều chuyển từ kho trung tâm, đơn hàng dự kiến giao sau 2-3 ngày làm việc (Miễn phí vận chuyển)'.</t>
+        </is>
+      </c>
+      <c r="G76" s="12" t="inlineStr">
+        <is>
+          <t>Nếu khách cần nhận gấp Camera trong 2h: Cho phép khách tick chọn 'Tách giao Camera trước, phụ kiện giao sau'.</t>
+        </is>
+      </c>
+      <c r="H76" s="13" t="inlineStr">
+        <is>
+          <t>Khi kho giao hàng tại địa chỉ của khách hết phụ kiện mua kèm, Kinh doanh muốn điều chuyển kho miễn phí hay thông báo khách đổi mẫu khác?</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="28" customHeight="1">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>PHẦN 17: 17. BÁN KÈM SAU ĐẶT HÀNG (POST-PURCHASE ONE-CLICK UPSELL) TẠI TRANG THÀNH CÔNG</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="n"/>
+      <c r="C77" s="5" t="n"/>
+      <c r="D77" s="5" t="n"/>
+      <c r="E77" s="5" t="n"/>
+      <c r="F77" s="5" t="n"/>
+      <c r="G77" s="5" t="n"/>
+      <c r="H77" s="5" t="n"/>
+    </row>
+    <row r="78" ht="70" customHeight="1">
+      <c r="A78" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>BR-01</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>17. Bán kèm Sau Đặt Hàng (Post-Purchase One-Click Upsell) tại Trang Thành Công</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>Khách hoàn tất thanh toán Camera mà quên chọn phụ kiện mua kèm</t>
+        </is>
+      </c>
+      <c r="E78" s="8" t="inlineStr">
+        <is>
+          <t>Khách đã bấm Đặt hàng thành công đơn Camera Play 4 và chuyển đến trang 'Cảm ơn / Đặt hàng thành công'.</t>
+        </is>
+      </c>
+      <c r="F78" s="8" t="inlineStr">
+        <is>
+          <t>Kích hoạt đồng hồ đếm ngược 5 phút tại trang Cảm ơn: 'Đặc quyền của bạn: Thêm 01 Charm Play 4 với giá ưu đãi 0đ vào đơn hàng vừa tạo (Miễn phí vận chuyển)'. Khách click [Thêm ngay], hệ thống tự động gộp vào đơn hàng vừa tạo trước khi đẩy sang kho WMS.</t>
+        </is>
+      </c>
+      <c r="G78" s="8" t="inlineStr">
+        <is>
+          <t>Sau 5 phút hoặc khi đơn hàng đã chuyển trạng thái 'Đang đóng gói', ưu đãi bổ sung này tự động hết hiệu lực.</t>
+        </is>
+      </c>
+      <c r="H78" s="9" t="inlineStr">
+        <is>
+          <t>Kinh doanh có đồng ý cho phép khách bổ sung phụ kiện mua kèm vào đơn hàng vừa tạo trong vòng 5 phút tại màn hình Cảm ơn không?</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="17">
+    <mergeCell ref="A70:H70"/>
     <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A77:H77"/>
     <mergeCell ref="A29:H29"/>
     <mergeCell ref="A57:H57"/>
+    <mergeCell ref="A73:H73"/>
     <mergeCell ref="A16:H16"/>
     <mergeCell ref="A51:H51"/>
     <mergeCell ref="A54:H54"/>
     <mergeCell ref="A63:H63"/>
     <mergeCell ref="A60:H60"/>
+    <mergeCell ref="A66:H66"/>
     <mergeCell ref="A44:H44"/>
     <mergeCell ref="A47:H47"/>
     <mergeCell ref="A5:H5"/>

</xml_diff>